<commit_message>
fix: wire widget capability chips to translations; park Nigeria language bundle
Nine capability-chip labels in the widget (intent/outcome chips, "General
guidance", "Routed to a person", the sources-count chip) were hardcoded
English despite matching label_* keys already existing translated in all
six languages — the exact "complete string table, dead call sites" failure
this product has hit before. INTENTS/OUTCOMES now carry a translation key
instead of literal text, resolved with T() at render time; two missing
keys (label_routed_to_person, n_sources/one_source with proper {n}
interpolation instead of string-concatenated pluralization) added across
all six languages. Verified live via Playwright in Swahili, Amharic and
English.

Also records a regional-focus decision: the Hausa/Yoruba/Igbo bundle is
parked (not cancelled) in favor of staying in East Africa, the region
Swahili already anchors, before a second regional jump to West Africa.
ADR-0019.
</commit_message>
<xml_diff>
--- a/review/Olink_Bank_Assist_language_review.xlsx
+++ b/review/Olink_Bank_Assist_language_review.xlsx
@@ -16,7 +16,7 @@
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'1. What the assistant says'!$A$1:$I$21</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'2. What it understands'!$A$1:$E$91</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'3. Buttons customers see'!$A$1:$I$50</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'3. Buttons customers see'!$A$1:$I$53</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'4. The staff panel'!$A$1:$I$270</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -752,7 +752,7 @@
       </c>
       <c r="C26" s="6" t="inlineStr">
         <is>
-          <t>338 strings in 5 languages</t>
+          <t>341 strings in 5 languages</t>
         </is>
       </c>
     </row>
@@ -3915,7 +3915,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I50"/>
+  <dimension ref="A1:I53"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
@@ -6000,7 +6000,7 @@
     <row r="49" ht="44" customHeight="1">
       <c r="A49" s="11" t="inlineStr">
         <is>
-          <t>today</t>
+          <t>label_routed_to_person</t>
         </is>
       </c>
       <c r="B49" s="11" t="inlineStr">
@@ -6010,32 +6010,32 @@
       </c>
       <c r="C49" s="11" t="inlineStr">
         <is>
-          <t>Today</t>
+          <t>Routed to a person</t>
         </is>
       </c>
       <c r="D49" s="12" t="inlineStr">
         <is>
-          <t>ዛሬ</t>
+          <t>ወደ ሰው ተላልፏል</t>
         </is>
       </c>
       <c r="E49" s="13" t="inlineStr">
         <is>
-          <t>Har'a</t>
+          <t>Gara namaatti dabarfameera</t>
         </is>
       </c>
       <c r="F49" s="12" t="inlineStr">
         <is>
-          <t>ሎሚ</t>
+          <t>ናብ ሰብ ተመሓላሊፉ</t>
         </is>
       </c>
       <c r="G49" s="13" t="inlineStr">
         <is>
-          <t>Maanta</t>
+          <t>Loo gudbiyay qof</t>
         </is>
       </c>
       <c r="H49" s="13" t="inlineStr">
         <is>
-          <t>Leo</t>
+          <t>Imeelekezwa kwa mtu</t>
         </is>
       </c>
       <c r="I49" s="14" t="inlineStr"/>
@@ -6043,48 +6043,177 @@
     <row r="50" ht="44" customHeight="1">
       <c r="A50" s="11" t="inlineStr">
         <is>
+          <t>n_sources</t>
+        </is>
+      </c>
+      <c r="B50" s="11" t="inlineStr">
+        <is>
+          <t>Button, label or placeholder in the chat window. Keep it short — it has to fit the same space as the English, on a phone.</t>
+        </is>
+      </c>
+      <c r="C50" s="11" t="inlineStr">
+        <is>
+          <t>{n} sources</t>
+        </is>
+      </c>
+      <c r="D50" s="12" t="inlineStr">
+        <is>
+          <t>{n} ምንጮች</t>
+        </is>
+      </c>
+      <c r="E50" s="13" t="inlineStr">
+        <is>
+          <t>Maddoota {n}</t>
+        </is>
+      </c>
+      <c r="F50" s="12" t="inlineStr">
+        <is>
+          <t>{n} ምንጭታት</t>
+        </is>
+      </c>
+      <c r="G50" s="13" t="inlineStr">
+        <is>
+          <t>{n} ilo</t>
+        </is>
+      </c>
+      <c r="H50" s="13" t="inlineStr">
+        <is>
+          <t>Vyanzo {n}</t>
+        </is>
+      </c>
+      <c r="I50" s="14" t="inlineStr"/>
+    </row>
+    <row r="51" ht="44" customHeight="1">
+      <c r="A51" s="11" t="inlineStr">
+        <is>
+          <t>one_source</t>
+        </is>
+      </c>
+      <c r="B51" s="11" t="inlineStr">
+        <is>
+          <t>Button, label or placeholder in the chat window. Keep it short — it has to fit the same space as the English, on a phone.</t>
+        </is>
+      </c>
+      <c r="C51" s="11" t="inlineStr">
+        <is>
+          <t>{n} source</t>
+        </is>
+      </c>
+      <c r="D51" s="12" t="inlineStr">
+        <is>
+          <t>{n} ምንጭ</t>
+        </is>
+      </c>
+      <c r="E51" s="13" t="inlineStr">
+        <is>
+          <t>Madda {n}</t>
+        </is>
+      </c>
+      <c r="F51" s="12" t="inlineStr">
+        <is>
+          <t>{n} ምንጪ</t>
+        </is>
+      </c>
+      <c r="G51" s="13" t="inlineStr">
+        <is>
+          <t>{n} il</t>
+        </is>
+      </c>
+      <c r="H51" s="13" t="inlineStr">
+        <is>
+          <t>Chanzo {n}</t>
+        </is>
+      </c>
+      <c r="I51" s="14" t="inlineStr"/>
+    </row>
+    <row r="52" ht="44" customHeight="1">
+      <c r="A52" s="11" t="inlineStr">
+        <is>
+          <t>today</t>
+        </is>
+      </c>
+      <c r="B52" s="11" t="inlineStr">
+        <is>
+          <t>Button, label or placeholder in the chat window. Keep it short — it has to fit the same space as the English, on a phone.</t>
+        </is>
+      </c>
+      <c r="C52" s="11" t="inlineStr">
+        <is>
+          <t>Today</t>
+        </is>
+      </c>
+      <c r="D52" s="12" t="inlineStr">
+        <is>
+          <t>ዛሬ</t>
+        </is>
+      </c>
+      <c r="E52" s="13" t="inlineStr">
+        <is>
+          <t>Har'a</t>
+        </is>
+      </c>
+      <c r="F52" s="12" t="inlineStr">
+        <is>
+          <t>ሎሚ</t>
+        </is>
+      </c>
+      <c r="G52" s="13" t="inlineStr">
+        <is>
+          <t>Maanta</t>
+        </is>
+      </c>
+      <c r="H52" s="13" t="inlineStr">
+        <is>
+          <t>Leo</t>
+        </is>
+      </c>
+      <c r="I52" s="14" t="inlineStr"/>
+    </row>
+    <row r="53" ht="44" customHeight="1">
+      <c r="A53" s="11" t="inlineStr">
+        <is>
           <t>yesterday</t>
         </is>
       </c>
-      <c r="B50" s="11" t="inlineStr">
+      <c r="B53" s="11" t="inlineStr">
         <is>
           <t>Button, label or placeholder in the chat window. Keep it short — it has to fit the same space as the English, on a phone.</t>
         </is>
       </c>
-      <c r="C50" s="11" t="inlineStr">
+      <c r="C53" s="11" t="inlineStr">
         <is>
           <t>Yesterday</t>
         </is>
       </c>
-      <c r="D50" s="12" t="inlineStr">
+      <c r="D53" s="12" t="inlineStr">
         <is>
           <t>ትናንት</t>
         </is>
       </c>
-      <c r="E50" s="13" t="inlineStr">
+      <c r="E53" s="13" t="inlineStr">
         <is>
           <t>Kaleessa</t>
         </is>
       </c>
-      <c r="F50" s="12" t="inlineStr">
+      <c r="F53" s="12" t="inlineStr">
         <is>
           <t>ትማሊ</t>
         </is>
       </c>
-      <c r="G50" s="13" t="inlineStr">
+      <c r="G53" s="13" t="inlineStr">
         <is>
           <t>Shalay</t>
         </is>
       </c>
-      <c r="H50" s="13" t="inlineStr">
+      <c r="H53" s="13" t="inlineStr">
         <is>
           <t>Jana</t>
         </is>
       </c>
-      <c r="I50" s="14" t="inlineStr"/>
+      <c r="I53" s="14" t="inlineStr"/>
     </row>
   </sheetData>
-  <autoFilter ref="A1:I50"/>
+  <autoFilter ref="A1:I53"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
feat: connect forms for the five channels that had none (#162)
The Channels page described seven channels and offered a way to switch on
two. Viber, WhatsApp, Messenger, Instagram and SMS each got a page
explaining the channel and then nothing to do about it, while the backend
routes had been written, tested and deployed the whole time.

Viber matters most of the five: its bot account is self-serve, so it was
the one channel a bank could have switched on that day and could not.

Meta's three share one panel — the app secret is optional once stored, so
adding Messenger in June does not mean retyping the credential WhatsApp
was connected with in March. SMS keeps its stored authorization header
when the field is left blank, and its inbound secret is held across the
reload that renders it.

41 new strings in six languages. test_channel_connect_ui.py walks
channels.CATALOGUE so an eighth channel cannot ship without a form.
</commit_message>
<xml_diff>
--- a/review/Olink_Bank_Assist_language_review.xlsx
+++ b/review/Olink_Bank_Assist_language_review.xlsx
@@ -17,7 +17,7 @@
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'1. What the assistant says'!$A$1:$I$23</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'2. What it understands'!$A$1:$E$91</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'3. Buttons customers see'!$A$1:$I$53</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'4. The staff panel'!$A$1:$I$417</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'4. The staff panel'!$A$1:$I$459</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -752,7 +752,7 @@
       </c>
       <c r="C26" s="6" t="inlineStr">
         <is>
-          <t>490 strings in 5 languages</t>
+          <t>532 strings in 5 languages</t>
         </is>
       </c>
     </row>
@@ -6302,7 +6302,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I417"/>
+  <dimension ref="A1:I459"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
@@ -24251,8 +24251,1814 @@
       </c>
       <c r="I417" s="14" t="inlineStr"/>
     </row>
+    <row r="418" ht="44" customHeight="1">
+      <c r="A418" s="11" t="inlineStr">
+        <is>
+          <t>chan_connect</t>
+        </is>
+      </c>
+      <c r="B418" s="11" t="inlineStr">
+        <is>
+          <t>Read by bank staff, not customers. Keep it short — it has to fit the same space as the English. Use the words your branch staff already use.</t>
+        </is>
+      </c>
+      <c r="C418" s="11" t="inlineStr">
+        <is>
+          <t>Connect</t>
+        </is>
+      </c>
+      <c r="D418" s="12" t="inlineStr">
+        <is>
+          <t>አገናኝ</t>
+        </is>
+      </c>
+      <c r="E418" s="13" t="inlineStr">
+        <is>
+          <t>Wal qunnamsiisi</t>
+        </is>
+      </c>
+      <c r="F418" s="12" t="inlineStr">
+        <is>
+          <t>ኣራኽብ</t>
+        </is>
+      </c>
+      <c r="G418" s="13" t="inlineStr">
+        <is>
+          <t>Ku xidhiidhi</t>
+        </is>
+      </c>
+      <c r="H418" s="13" t="inlineStr">
+        <is>
+          <t>Unganisha</t>
+        </is>
+      </c>
+      <c r="I418" s="14" t="inlineStr"/>
+    </row>
+    <row r="419" ht="44" customHeight="1">
+      <c r="A419" s="11" t="inlineStr">
+        <is>
+          <t>chan_update</t>
+        </is>
+      </c>
+      <c r="B419" s="11" t="inlineStr">
+        <is>
+          <t>Read by bank staff, not customers. Keep it short — it has to fit the same space as the English. Use the words your branch staff already use.</t>
+        </is>
+      </c>
+      <c r="C419" s="11" t="inlineStr">
+        <is>
+          <t>Update</t>
+        </is>
+      </c>
+      <c r="D419" s="12" t="inlineStr">
+        <is>
+          <t>አዘምን</t>
+        </is>
+      </c>
+      <c r="E419" s="13" t="inlineStr">
+        <is>
+          <t>Haaromsi</t>
+        </is>
+      </c>
+      <c r="F419" s="12" t="inlineStr">
+        <is>
+          <t>ኣሐድስ</t>
+        </is>
+      </c>
+      <c r="G419" s="13" t="inlineStr">
+        <is>
+          <t>Cusboonaysii</t>
+        </is>
+      </c>
+      <c r="H419" s="13" t="inlineStr">
+        <is>
+          <t>Sasisha</t>
+        </is>
+      </c>
+      <c r="I419" s="14" t="inlineStr"/>
+    </row>
+    <row r="420" ht="44" customHeight="1">
+      <c r="A420" s="11" t="inlineStr">
+        <is>
+          <t>chan_copy</t>
+        </is>
+      </c>
+      <c r="B420" s="11" t="inlineStr">
+        <is>
+          <t>Read by bank staff, not customers. Keep it short — it has to fit the same space as the English. Use the words your branch staff already use.</t>
+        </is>
+      </c>
+      <c r="C420" s="11" t="inlineStr">
+        <is>
+          <t>Copy</t>
+        </is>
+      </c>
+      <c r="D420" s="12" t="inlineStr">
+        <is>
+          <t>ቅዳ</t>
+        </is>
+      </c>
+      <c r="E420" s="13" t="inlineStr">
+        <is>
+          <t>Garagalchi</t>
+        </is>
+      </c>
+      <c r="F420" s="12" t="inlineStr">
+        <is>
+          <t>ቅዳሕ</t>
+        </is>
+      </c>
+      <c r="G420" s="13" t="inlineStr">
+        <is>
+          <t>Koobi</t>
+        </is>
+      </c>
+      <c r="H420" s="13" t="inlineStr">
+        <is>
+          <t>Nakili</t>
+        </is>
+      </c>
+      <c r="I420" s="14" t="inlineStr"/>
+    </row>
+    <row r="421" ht="44" customHeight="1">
+      <c r="A421" s="11" t="inlineStr">
+        <is>
+          <t>chan_copied</t>
+        </is>
+      </c>
+      <c r="B421" s="11" t="inlineStr">
+        <is>
+          <t>Read by bank staff, not customers. Keep it short — it has to fit the same space as the English. Use the words your branch staff already use.</t>
+        </is>
+      </c>
+      <c r="C421" s="11" t="inlineStr">
+        <is>
+          <t>Copied</t>
+        </is>
+      </c>
+      <c r="D421" s="12" t="inlineStr">
+        <is>
+          <t>ተቀድቷል</t>
+        </is>
+      </c>
+      <c r="E421" s="13" t="inlineStr">
+        <is>
+          <t>Garagalfameera</t>
+        </is>
+      </c>
+      <c r="F421" s="12" t="inlineStr">
+        <is>
+          <t>ተቐዲሑ</t>
+        </is>
+      </c>
+      <c r="G421" s="13" t="inlineStr">
+        <is>
+          <t>Waa la koobiyeeyay</t>
+        </is>
+      </c>
+      <c r="H421" s="13" t="inlineStr">
+        <is>
+          <t>Imenakiliwa</t>
+        </is>
+      </c>
+      <c r="I421" s="14" t="inlineStr"/>
+    </row>
+    <row r="422" ht="44" customHeight="1">
+      <c r="A422" s="11" t="inlineStr">
+        <is>
+          <t>chan_web_title</t>
+        </is>
+      </c>
+      <c r="B422" s="11" t="inlineStr">
+        <is>
+          <t>Read by bank staff, not customers. Keep it short — it has to fit the same space as the English. Use the words your branch staff already use.</t>
+        </is>
+      </c>
+      <c r="C422" s="11" t="inlineStr">
+        <is>
+          <t>Put the widget on your website</t>
+        </is>
+      </c>
+      <c r="D422" s="12" t="inlineStr">
+        <is>
+          <t>መስኮቱን በድረ-ገጽዎ ላይ ያስቀምጡ</t>
+        </is>
+      </c>
+      <c r="E422" s="13" t="inlineStr">
+        <is>
+          <t>Widjetii kana marsariitii keessan irra kaa'aa</t>
+        </is>
+      </c>
+      <c r="F422" s="12" t="inlineStr">
+        <is>
+          <t>ነቲ መስኮት ኣብ መርበብ ሓበሬታኹም ኣቐምጡ</t>
+        </is>
+      </c>
+      <c r="G422" s="13" t="inlineStr">
+        <is>
+          <t>Widget-ka geli degelkaaga</t>
+        </is>
+      </c>
+      <c r="H422" s="13" t="inlineStr">
+        <is>
+          <t>Weka kidirisha kwenye tovuti yako</t>
+        </is>
+      </c>
+      <c r="I422" s="14" t="inlineStr"/>
+    </row>
+    <row r="423" ht="44" customHeight="1">
+      <c r="A423" s="11" t="inlineStr">
+        <is>
+          <t>chan_web_help</t>
+        </is>
+      </c>
+      <c r="B423" s="11" t="inlineStr">
+        <is>
+          <t>Read by bank staff, not customers. Keep it short — it has to fit the same space as the English. Use the words your branch staff already use.</t>
+        </is>
+      </c>
+      <c r="C423" s="11" t="inlineStr">
+        <is>
+          <t>Paste this once, before the closing &lt;/body&gt; tag. It adds a chat button in your own colour and loads nothing until a visitor opens it.</t>
+        </is>
+      </c>
+      <c r="D423" s="12" t="inlineStr">
+        <is>
+          <t>ይህን አንድ ጊዜ፣ ከ&lt;/body&gt; መዝጊያ በፊት ይለጥፉ። በራስዎ ቀለም የውይይት አዝራር ይጨምራል፤ ጎብኚ እስኪከፍተው ድረስ ምንም አይጫንም።</t>
+        </is>
+      </c>
+      <c r="E423" s="13" t="inlineStr">
+        <is>
+          <t>Kana yeroo tokko, dura &lt;/body&gt; cufaa maxxansaa. Halluu keessaniin qabduu chat dabala, hanga daawwataan banutti homaa hin fe'u.</t>
+        </is>
+      </c>
+      <c r="F423" s="12" t="inlineStr">
+        <is>
+          <t>ነዚ ሓደ ግዜ፣ ቅድሚ እቲ ዝዓጹ &lt;/body&gt; ለጥፍዎ። ብሕብርኹም መጠወቒ ዝርርብ ይውስኽ፣ በጻሒ ክሳብ ዝኸፍቶ ገለ ኣይጽዕንን።</t>
+        </is>
+      </c>
+      <c r="G423" s="13" t="inlineStr">
+        <is>
+          <t>Mid kaliya ku dheji, ka hor summadda xidhitaanka ee &lt;/body&gt;. Wuxuu ku darayaa badhan sheeko oo midabkaaga ah, waxbana ma raro ilaa booqde furo.</t>
+        </is>
+      </c>
+      <c r="H423" s="13" t="inlineStr">
+        <is>
+          <t>Bandika hii mara moja, kabla ya lebo ya kufunga &lt;/body&gt;. Inaongeza kitufe cha mazungumzo kwa rangi yako na haipakii chochote hadi mtembeleaji akifungue.</t>
+        </is>
+      </c>
+      <c r="I423" s="14" t="inlineStr"/>
+    </row>
+    <row r="424" ht="44" customHeight="1">
+      <c r="A424" s="11" t="inlineStr">
+        <is>
+          <t>chan_telegram_title</t>
+        </is>
+      </c>
+      <c r="B424" s="11" t="inlineStr">
+        <is>
+          <t>Read by bank staff, not customers. Keep it short — it has to fit the same space as the English. Use the words your branch staff already use.</t>
+        </is>
+      </c>
+      <c r="C424" s="11" t="inlineStr">
+        <is>
+          <t>Connect your bot</t>
+        </is>
+      </c>
+      <c r="D424" s="12" t="inlineStr">
+        <is>
+          <t>ቦትዎን ያገናኙ</t>
+        </is>
+      </c>
+      <c r="E424" s="13" t="inlineStr">
+        <is>
+          <t>Boot keessan wal qunnamsiisaa</t>
+        </is>
+      </c>
+      <c r="F424" s="12" t="inlineStr">
+        <is>
+          <t>ቦትኩም ኣራኽቡ</t>
+        </is>
+      </c>
+      <c r="G424" s="13" t="inlineStr">
+        <is>
+          <t>Ku xidhiidhi bot-kaaga</t>
+        </is>
+      </c>
+      <c r="H424" s="13" t="inlineStr">
+        <is>
+          <t>Unganisha boti yako</t>
+        </is>
+      </c>
+      <c r="I424" s="14" t="inlineStr"/>
+    </row>
+    <row r="425" ht="44" customHeight="1">
+      <c r="A425" s="11" t="inlineStr">
+        <is>
+          <t>chan_telegram_help</t>
+        </is>
+      </c>
+      <c r="B425" s="11" t="inlineStr">
+        <is>
+          <t>Read by bank staff, not customers. Keep it short — it has to fit the same space as the English. Use the words your branch staff already use.</t>
+        </is>
+      </c>
+      <c r="C425" s="11" t="inlineStr">
+        <is>
+          <t>Message @BotFather on Telegram, send /newbot, and paste the token it gives you.</t>
+        </is>
+      </c>
+      <c r="D425" s="12" t="inlineStr">
+        <is>
+          <t>በቴሌግራም ላይ @BotFather ን ያነጋግሩ፣ /newbot ይላኩ፣ የሚሰጥዎትን ቶከን እዚህ ይለጥፉ።</t>
+        </is>
+      </c>
+      <c r="E425" s="13" t="inlineStr">
+        <is>
+          <t>Telegram irratti @BotFather dubbisaa, /newbot ergaa, tokeenii isaan isinii kennan asitti maxxansaa.</t>
+        </is>
+      </c>
+      <c r="F425" s="12" t="inlineStr">
+        <is>
+          <t>ኣብ ቴለግራም ንmy@BotFather ተወከሱ፣ /newbot ስደዱ፣ እቲ ዝህበኩም ቶከን ኣብዚ ለጥፍዎ።</t>
+        </is>
+      </c>
+      <c r="G425" s="13" t="inlineStr">
+        <is>
+          <t>Telegram ku fariin dir @BotFather, dir /newbot, kadibna halkan ku dheji token-ka ay ku siiyaan.</t>
+        </is>
+      </c>
+      <c r="H425" s="13" t="inlineStr">
+        <is>
+          <t>Tuma ujumbe kwa @BotFather kwenye Telegram, tuma /newbot, kisha bandika tokeni anayokupa hapa.</t>
+        </is>
+      </c>
+      <c r="I425" s="14" t="inlineStr"/>
+    </row>
+    <row r="426" ht="44" customHeight="1">
+      <c r="A426" s="11" t="inlineStr">
+        <is>
+          <t>chan_telegram_placeholder</t>
+        </is>
+      </c>
+      <c r="B426" s="11" t="inlineStr">
+        <is>
+          <t>Read by bank staff, not customers. Keep it short — it has to fit the same space as the English. Use the words your branch staff already use.</t>
+        </is>
+      </c>
+      <c r="C426" s="11" t="inlineStr">
+        <is>
+          <t>Bot token from @BotFather</t>
+        </is>
+      </c>
+      <c r="D426" s="12" t="inlineStr">
+        <is>
+          <t>ከ@BotFather የተገኘ የቦት ቶከን</t>
+        </is>
+      </c>
+      <c r="E426" s="13" t="inlineStr">
+        <is>
+          <t>Tokeenii boot @BotFather irraa</t>
+        </is>
+      </c>
+      <c r="F426" s="12" t="inlineStr">
+        <is>
+          <t>ካብ @BotFather ዝተረኽበ ቶከን ቦት</t>
+        </is>
+      </c>
+      <c r="G426" s="13" t="inlineStr">
+        <is>
+          <t>Token bot ah oo ka yimid @BotFather</t>
+        </is>
+      </c>
+      <c r="H426" s="13" t="inlineStr">
+        <is>
+          <t>Tokeni ya boti kutoka @BotFather</t>
+        </is>
+      </c>
+      <c r="I426" s="14" t="inlineStr"/>
+    </row>
+    <row r="427" ht="44" customHeight="1">
+      <c r="A427" s="11" t="inlineStr">
+        <is>
+          <t>chan_replaces_current</t>
+        </is>
+      </c>
+      <c r="B427" s="11" t="inlineStr">
+        <is>
+          <t>Read by bank staff, not customers. Keep it short — it has to fit the same space as the English. Use the words your branch staff already use.</t>
+        </is>
+      </c>
+      <c r="C427" s="11" t="inlineStr">
+        <is>
+          <t>Entering a new token replaces the current connection.</t>
+        </is>
+      </c>
+      <c r="D427" s="12" t="inlineStr">
+        <is>
+          <t>አዲስ ቶከን ማስገባት አሁን ያለውን ግንኙነት ይተካል።</t>
+        </is>
+      </c>
+      <c r="E427" s="13" t="inlineStr">
+        <is>
+          <t>Tokeenii haaraa galchuun walqunnamtii ammaa bakka bu'a.</t>
+        </is>
+      </c>
+      <c r="F427" s="12" t="inlineStr">
+        <is>
+          <t>ሓድሽ ቶከን ምእታው ነቲ ህሉው ርክብ ይትክኦ።</t>
+        </is>
+      </c>
+      <c r="G427" s="13" t="inlineStr">
+        <is>
+          <t>Token cusub oo la geliyo wuxuu beddelayaa xidhiidhka hadda jira.</t>
+        </is>
+      </c>
+      <c r="H427" s="13" t="inlineStr">
+        <is>
+          <t>Kuweka tokeni mpya kunabadilisha muunganisho uliopo.</t>
+        </is>
+      </c>
+      <c r="I427" s="14" t="inlineStr"/>
+    </row>
+    <row r="428" ht="44" customHeight="1">
+      <c r="A428" s="11" t="inlineStr">
+        <is>
+          <t>chan_viber_title</t>
+        </is>
+      </c>
+      <c r="B428" s="11" t="inlineStr">
+        <is>
+          <t>Read by bank staff, not customers. Keep it short — it has to fit the same space as the English. Use the words your branch staff already use.</t>
+        </is>
+      </c>
+      <c r="C428" s="11" t="inlineStr">
+        <is>
+          <t>Connect your Viber bot</t>
+        </is>
+      </c>
+      <c r="D428" s="12" t="inlineStr">
+        <is>
+          <t>የቫይበር ቦትዎን ያገናኙ</t>
+        </is>
+      </c>
+      <c r="E428" s="13" t="inlineStr">
+        <is>
+          <t>Boot Viber keessan wal qunnamsiisaa</t>
+        </is>
+      </c>
+      <c r="F428" s="12" t="inlineStr">
+        <is>
+          <t>ቦት ቫይበርኩም ኣራኽቡ</t>
+        </is>
+      </c>
+      <c r="G428" s="13" t="inlineStr">
+        <is>
+          <t>Ku xidhiidhi bot-kaaga Viber</t>
+        </is>
+      </c>
+      <c r="H428" s="13" t="inlineStr">
+        <is>
+          <t>Unganisha boti yako ya Viber</t>
+        </is>
+      </c>
+      <c r="I428" s="14" t="inlineStr"/>
+    </row>
+    <row r="429" ht="44" customHeight="1">
+      <c r="A429" s="11" t="inlineStr">
+        <is>
+          <t>chan_viber_help</t>
+        </is>
+      </c>
+      <c r="B429" s="11" t="inlineStr">
+        <is>
+          <t>Read by bank staff, not customers. Keep it short — it has to fit the same space as the English. Use the words your branch staff already use.</t>
+        </is>
+      </c>
+      <c r="C429" s="11" t="inlineStr">
+        <is>
+          <t>Create a bot account at partners.viber.com. It is self-serve and issues the authentication token straight away — paste it here and we register the webhook for you.</t>
+        </is>
+      </c>
+      <c r="D429" s="12" t="inlineStr">
+        <is>
+          <t>በ partners.viber.com ላይ የቦት መለያ ይፍጠሩ። ራስን የሚያገለግል ነው፤ የማረጋገጫ ቶከኑን ወዲያውኑ ይሰጣል — እዚህ ይለጥፉት፤ ድረ-መንጠቆውን እኛ እንመዘግባለን።</t>
+        </is>
+      </c>
+      <c r="E429" s="13" t="inlineStr">
+        <is>
+          <t>partners.viber.com irratti akkaawuntii boot uumaa. Ofii keessaniin raawwatama, tokeenii mirkaneessaa battalumatti kenna — asitti maxxansaa, webhook isa nuti galmeessina.</t>
+        </is>
+      </c>
+      <c r="F429" s="12" t="inlineStr">
+        <is>
+          <t>ኣብ partners.viber.com ኣካውንት ቦት ፍጠሩ። ባዕልኹም እትገብርዎ እዩ፣ ቶከን መረጋገጺ ብቕጽበት ይህብ — ኣብዚ ለጥፍዎ፣ ነቲ ወብ-ሁክ ንሕና ንምዝግቦ።</t>
+        </is>
+      </c>
+      <c r="G429" s="13" t="inlineStr">
+        <is>
+          <t>Akoon bot ah ka samayso partners.viber.com. Waa mid aad adigu samayn karto, isla markaana ku siinaya token-ka xaqiijinta — halkan ku dheji, annagana webhook-ga waan kuu diiwaan gelinaynaa.</t>
+        </is>
+      </c>
+      <c r="H429" s="13" t="inlineStr">
+        <is>
+          <t>Fungua akaunti ya boti kwenye partners.viber.com. Ni ya kujihudumia na inatoa tokeni ya uthibitisho papo hapo — ibandike hapa na sisi tutasajili webhook kwa niaba yako.</t>
+        </is>
+      </c>
+      <c r="I429" s="14" t="inlineStr"/>
+    </row>
+    <row r="430" ht="44" customHeight="1">
+      <c r="A430" s="11" t="inlineStr">
+        <is>
+          <t>chan_viber_placeholder</t>
+        </is>
+      </c>
+      <c r="B430" s="11" t="inlineStr">
+        <is>
+          <t>Read by bank staff, not customers. Keep it short — it has to fit the same space as the English. Use the words your branch staff already use.</t>
+        </is>
+      </c>
+      <c r="C430" s="11" t="inlineStr">
+        <is>
+          <t>Authentication token from partners.viber.com</t>
+        </is>
+      </c>
+      <c r="D430" s="12" t="inlineStr">
+        <is>
+          <t>ከ partners.viber.com የተገኘ የማረጋገጫ ቶከን</t>
+        </is>
+      </c>
+      <c r="E430" s="13" t="inlineStr">
+        <is>
+          <t>Tokeenii mirkaneessaa partners.viber.com irraa</t>
+        </is>
+      </c>
+      <c r="F430" s="12" t="inlineStr">
+        <is>
+          <t>ካብ partners.viber.com ዝተረኽበ ቶከን መረጋገጺ</t>
+        </is>
+      </c>
+      <c r="G430" s="13" t="inlineStr">
+        <is>
+          <t>Token xaqiijin ah oo ka yimid partners.viber.com</t>
+        </is>
+      </c>
+      <c r="H430" s="13" t="inlineStr">
+        <is>
+          <t>Tokeni ya uthibitisho kutoka partners.viber.com</t>
+        </is>
+      </c>
+      <c r="I430" s="14" t="inlineStr"/>
+    </row>
+    <row r="431" ht="44" customHeight="1">
+      <c r="A431" s="11" t="inlineStr">
+        <is>
+          <t>chan_viber_connected</t>
+        </is>
+      </c>
+      <c r="B431" s="11" t="inlineStr">
+        <is>
+          <t>Read by bank staff, not customers. Keep it short — it has to fit the same space as the English. Use the words your branch staff already use.</t>
+        </is>
+      </c>
+      <c r="C431" s="11" t="inlineStr">
+        <is>
+          <t>Viber connected</t>
+        </is>
+      </c>
+      <c r="D431" s="12" t="inlineStr">
+        <is>
+          <t>ቫይበር ተገናኝቷል</t>
+        </is>
+      </c>
+      <c r="E431" s="13" t="inlineStr">
+        <is>
+          <t>Viber wal qunnameera</t>
+        </is>
+      </c>
+      <c r="F431" s="12" t="inlineStr">
+        <is>
+          <t>ቫይበር ተራኺቡ</t>
+        </is>
+      </c>
+      <c r="G431" s="13" t="inlineStr">
+        <is>
+          <t>Viber waa la xidhiidhiyay</t>
+        </is>
+      </c>
+      <c r="H431" s="13" t="inlineStr">
+        <is>
+          <t>Viber imeunganishwa</t>
+        </is>
+      </c>
+      <c r="I431" s="14" t="inlineStr"/>
+    </row>
+    <row r="432" ht="44" customHeight="1">
+      <c r="A432" s="11" t="inlineStr">
+        <is>
+          <t>chan_meta_title</t>
+        </is>
+      </c>
+      <c r="B432" s="11" t="inlineStr">
+        <is>
+          <t>Read by bank staff, not customers. Keep it short — it has to fit the same space as the English. Use the words your branch staff already use.</t>
+        </is>
+      </c>
+      <c r="C432" s="11" t="inlineStr">
+        <is>
+          <t>Connect through Meta</t>
+        </is>
+      </c>
+      <c r="D432" s="12" t="inlineStr">
+        <is>
+          <t>በሜታ በኩል ያገናኙ</t>
+        </is>
+      </c>
+      <c r="E432" s="13" t="inlineStr">
+        <is>
+          <t>Meta karaa wal qunnamsiisaa</t>
+        </is>
+      </c>
+      <c r="F432" s="12" t="inlineStr">
+        <is>
+          <t>ብሜታ ኣቢልኩም ኣራኽቡ</t>
+        </is>
+      </c>
+      <c r="G432" s="13" t="inlineStr">
+        <is>
+          <t>Ku xidhiidh Meta</t>
+        </is>
+      </c>
+      <c r="H432" s="13" t="inlineStr">
+        <is>
+          <t>Unganisha kupitia Meta</t>
+        </is>
+      </c>
+      <c r="I432" s="14" t="inlineStr"/>
+    </row>
+    <row r="433" ht="44" customHeight="1">
+      <c r="A433" s="11" t="inlineStr">
+        <is>
+          <t>chan_meta_help</t>
+        </is>
+      </c>
+      <c r="B433" s="11" t="inlineStr">
+        <is>
+          <t>Read by bank staff, not customers. Keep it short — it has to fit the same space as the English. Use the words your branch staff already use.</t>
+        </is>
+      </c>
+      <c r="C433" s="11" t="inlineStr">
+        <is>
+          <t>WhatsApp, Messenger and Instagram all run through one Meta app. Connect the app once, then add the credential for whichever product Meta has approved — the others keep working untouched.</t>
+        </is>
+      </c>
+      <c r="D433" s="12" t="inlineStr">
+        <is>
+          <t>ዋትስአፕ፣ መሴንጀርና ኢንስታግራም ሁሉም በአንድ የሜታ መተግበሪያ በኩል ይሠራሉ። መተግበሪያውን አንድ ጊዜ ያገናኙ፤ ከዚያ ሜታ ላጸደቀው ምርት መረጃውን ይጨምሩ — ሌሎቹ ሳይነኩ መስራታቸውን ይቀጥላሉ።</t>
+        </is>
+      </c>
+      <c r="E433" s="13" t="inlineStr">
+        <is>
+          <t>WhatsApp, Messenger fi Instagram hundi appii Meta tokkoon hojjetu. Appii sana yeroo tokko wal qunnamsiisaa, achiis oomisha Meta mirkaneesseef ragaa dabalaa — kaan osoo hin tuqamin hojjechuu itti fufu.</t>
+        </is>
+      </c>
+      <c r="F433" s="12" t="inlineStr">
+        <is>
+          <t>ዋትስኣፕ፣ መሰንጀርን ኢንስታግራምን ኩሎም ብሓደ ኣፕ ሜታ እዮም ዝሰርሑ። ነቲ ኣፕ ሓንሳብ ኣራኽቡ፣ ደሓር ንዝኾነ ሜታ ዘጽደቖ ውጽኢት ሓበሬታ ወስኹ — እቶም ካልኦት ከይተተንከፉ ይቕጽሉ።</t>
+        </is>
+      </c>
+      <c r="G433" s="13" t="inlineStr">
+        <is>
+          <t>WhatsApp, Messenger iyo Instagram dhammaantood waxay ku shaqeeyaan hal app oo Meta ah. Hal mar ku xidhiidhi app-ka, kadibna ku dar aqoonsiga alaabta Meta ansixisay — kuwa kalena way sii shaqaynayaan iyagoo aan la taaban.</t>
+        </is>
+      </c>
+      <c r="H433" s="13" t="inlineStr">
+        <is>
+          <t>WhatsApp, Messenger na Instagram vyote hupitia programu moja ya Meta. Unganisha programu mara moja, kisha ongeza kitambulisho cha bidhaa yoyote ambayo Meta imeidhinisha — nyingine zinaendelea kufanya kazi bila kuguswa.</t>
+        </is>
+      </c>
+      <c r="I433" s="14" t="inlineStr"/>
+    </row>
+    <row r="434" ht="44" customHeight="1">
+      <c r="A434" s="11" t="inlineStr">
+        <is>
+          <t>chan_meta_app_secret</t>
+        </is>
+      </c>
+      <c r="B434" s="11" t="inlineStr">
+        <is>
+          <t>Read by bank staff, not customers. Keep it short — it has to fit the same space as the English. Use the words your branch staff already use.</t>
+        </is>
+      </c>
+      <c r="C434" s="11" t="inlineStr">
+        <is>
+          <t>App secret</t>
+        </is>
+      </c>
+      <c r="D434" s="12" t="inlineStr">
+        <is>
+          <t>የመተግበሪያ ሚስጥር</t>
+        </is>
+      </c>
+      <c r="E434" s="13" t="inlineStr">
+        <is>
+          <t>Iccitii appii</t>
+        </is>
+      </c>
+      <c r="F434" s="12" t="inlineStr">
+        <is>
+          <t>ምስጢር ኣፕ</t>
+        </is>
+      </c>
+      <c r="G434" s="13" t="inlineStr">
+        <is>
+          <t>Sirta app-ka</t>
+        </is>
+      </c>
+      <c r="H434" s="13" t="inlineStr">
+        <is>
+          <t>Siri ya programu</t>
+        </is>
+      </c>
+      <c r="I434" s="14" t="inlineStr"/>
+    </row>
+    <row r="435" ht="44" customHeight="1">
+      <c r="A435" s="11" t="inlineStr">
+        <is>
+          <t>chan_meta_app_secret_help</t>
+        </is>
+      </c>
+      <c r="B435" s="11" t="inlineStr">
+        <is>
+          <t>Read by bank staff, not customers. Keep it short — it has to fit the same space as the English. Use the words your branch staff already use.</t>
+        </is>
+      </c>
+      <c r="C435" s="11" t="inlineStr">
+        <is>
+          <t>From your Meta app's Basic settings. It is what proves a delivery really came from Meta, so nothing on these three channels works without it.</t>
+        </is>
+      </c>
+      <c r="D435" s="12" t="inlineStr">
+        <is>
+          <t>ከሜታ መተግበሪያዎ Basic ቅንብሮች። አንድ መልእክት በእውነት ከሜታ መምጣቱን የሚያረጋግጥ ነው፤ ስለዚህ ያለሱ በእነዚህ ሦስት መስመሮች ምንም አይሠራም።</t>
+        </is>
+      </c>
+      <c r="E435" s="13" t="inlineStr">
+        <is>
+          <t>Qindaa'ina Basic appii Meta keessanii irraa. Ergaan dhugumatti Meta irraa dhufuu isaa kan mirkaneessu isa, kanaafuu isa malee karaawwan sadan kanarratti homtuu hin hojjetu.</t>
+        </is>
+      </c>
+      <c r="F435" s="12" t="inlineStr">
+        <is>
+          <t>ካብ Basic ቅንብራት ኣፕ ሜታኹም። ሓደ መልእኽቲ ብሓቂ ካብ ሜታ ምምጽኡ ዘረጋግጽ እዩ፣ ስለዚ ብዘይኡ ኣብዘን ሰለስተ መስመራት ገለ ኣይሰርሕን።</t>
+        </is>
+      </c>
+      <c r="G435" s="13" t="inlineStr">
+        <is>
+          <t>Ka soo qaad goobaha Basic ee app-kaaga Meta. Waa waxa caddaynaya in fariin dhab ahaan Meta ka timid, sidaas darteed la'aanteed saddexdan kanaal waxba kuma shaqeeyaan.</t>
+        </is>
+      </c>
+      <c r="H435" s="13" t="inlineStr">
+        <is>
+          <t>Kutoka mipangilio ya Basic ya programu yako ya Meta. Ndiyo inayothibitisha kuwa ujumbe umetoka kweli Meta, kwa hivyo bila hiyo hakuna kinachofanya kazi kwenye njia hizi tatu.</t>
+        </is>
+      </c>
+      <c r="I435" s="14" t="inlineStr"/>
+    </row>
+    <row r="436" ht="44" customHeight="1">
+      <c r="A436" s="11" t="inlineStr">
+        <is>
+          <t>chan_meta_secret_stored</t>
+        </is>
+      </c>
+      <c r="B436" s="11" t="inlineStr">
+        <is>
+          <t>Read by bank staff, not customers. Keep it short — it has to fit the same space as the English. Use the words your branch staff already use.</t>
+        </is>
+      </c>
+      <c r="C436" s="11" t="inlineStr">
+        <is>
+          <t>An app secret is already stored. Leave this blank to keep it.</t>
+        </is>
+      </c>
+      <c r="D436" s="12" t="inlineStr">
+        <is>
+          <t>የመተግበሪያ ሚስጥር አስቀድሞ ተቀምጧል። ለማቆየት ይህን ባዶ ይተዉት።</t>
+        </is>
+      </c>
+      <c r="E436" s="13" t="inlineStr">
+        <is>
+          <t>Iccitiin appii duraanuu olkaa'ameera. Isa tursiisuuf kana duwwaa dhiisaa.</t>
+        </is>
+      </c>
+      <c r="F436" s="12" t="inlineStr">
+        <is>
+          <t>ምስጢር ኣፕ ድሮ ተቐሚጡ ኣሎ። ንምዕቃቡ ነዚ ባዶ ግደፍዎ።</t>
+        </is>
+      </c>
+      <c r="G436" s="13" t="inlineStr">
+        <is>
+          <t>Sir app ah horeyba waa la keydiyay. Si aad u hayso, banaan uga tag.</t>
+        </is>
+      </c>
+      <c r="H436" s="13" t="inlineStr">
+        <is>
+          <t>Siri ya programu tayari imehifadhiwa. Iache wazi ili kuiweka.</t>
+        </is>
+      </c>
+      <c r="I436" s="14" t="inlineStr"/>
+    </row>
+    <row r="437" ht="44" customHeight="1">
+      <c r="A437" s="11" t="inlineStr">
+        <is>
+          <t>chan_meta_paste_title</t>
+        </is>
+      </c>
+      <c r="B437" s="11" t="inlineStr">
+        <is>
+          <t>Read by bank staff, not customers. Keep it short — it has to fit the same space as the English. Use the words your branch staff already use.</t>
+        </is>
+      </c>
+      <c r="C437" s="11" t="inlineStr">
+        <is>
+          <t>Paste these into Meta</t>
+        </is>
+      </c>
+      <c r="D437" s="12" t="inlineStr">
+        <is>
+          <t>እነዚህን ወደ ሜታ ይለጥፉ</t>
+        </is>
+      </c>
+      <c r="E437" s="13" t="inlineStr">
+        <is>
+          <t>Kanneen Meta keessatti maxxansaa</t>
+        </is>
+      </c>
+      <c r="F437" s="12" t="inlineStr">
+        <is>
+          <t>እዚኦም ናብ ሜታ ለጥፍዎም</t>
+        </is>
+      </c>
+      <c r="G437" s="13" t="inlineStr">
+        <is>
+          <t>Kuwan ku dheji Meta</t>
+        </is>
+      </c>
+      <c r="H437" s="13" t="inlineStr">
+        <is>
+          <t>Bandika hizi kwenye Meta</t>
+        </is>
+      </c>
+      <c r="I437" s="14" t="inlineStr"/>
+    </row>
+    <row r="438" ht="44" customHeight="1">
+      <c r="A438" s="11" t="inlineStr">
+        <is>
+          <t>chan_meta_paste_help</t>
+        </is>
+      </c>
+      <c r="B438" s="11" t="inlineStr">
+        <is>
+          <t>Read by bank staff, not customers. Keep it short — it has to fit the same space as the English. Use the words your branch staff already use.</t>
+        </is>
+      </c>
+      <c r="C438" s="11" t="inlineStr">
+        <is>
+          <t>In your Meta app under Webhooks, use these two values, then subscribe to the messages events for each product you are switching on.</t>
+        </is>
+      </c>
+      <c r="D438" s="12" t="inlineStr">
+        <is>
+          <t>በሜታ መተግበሪያዎ ውስጥ በ Webhooks ስር እነዚህን ሁለት እሴቶች ይጠቀሙ፤ ከዚያ ለሚያበሩት ለእያንዳንዱ ምርት የ messages ክስተቶችን ይመዝገቡ።</t>
+        </is>
+      </c>
+      <c r="E438" s="13" t="inlineStr">
+        <is>
+          <t>Appii Meta keessan keessatti Webhooks jalatti gatiiwwan lamaan kana fayyadamaa, achiis oomisha banaa jirtan hundaaf taateewwan messages jedhamanitti galmaa'aa.</t>
+        </is>
+      </c>
+      <c r="F438" s="12" t="inlineStr">
+        <is>
+          <t>ኣብ ኣፕ ሜታኹም ኣብ ትሕቲ Webhooks ነዞም ክልተ ዋጋታት ተጠቐሙ፣ ደሓር ንዝኸፍትዎ ነፍሲ ወከፍ ውጽኢት ናይ messages ፍጻመታት ተመዝገቡ።</t>
+        </is>
+      </c>
+      <c r="G438" s="13" t="inlineStr">
+        <is>
+          <t>App-kaaga Meta ee hoosta Webhooks, isticmaal labadan qiyam, kadibna isku diiwaangeli dhacdooyinka messages ee alaab kasta oo aad shidayso.</t>
+        </is>
+      </c>
+      <c r="H438" s="13" t="inlineStr">
+        <is>
+          <t>Katika programu yako ya Meta chini ya Webhooks, tumia thamani hizi mbili, kisha jiandikishe kwa matukio ya messages kwa kila bidhaa unayowasha.</t>
+        </is>
+      </c>
+      <c r="I438" s="14" t="inlineStr"/>
+    </row>
+    <row r="439" ht="44" customHeight="1">
+      <c r="A439" s="11" t="inlineStr">
+        <is>
+          <t>chan_callback_url</t>
+        </is>
+      </c>
+      <c r="B439" s="11" t="inlineStr">
+        <is>
+          <t>Read by bank staff, not customers. Keep it short — it has to fit the same space as the English. Use the words your branch staff already use.</t>
+        </is>
+      </c>
+      <c r="C439" s="11" t="inlineStr">
+        <is>
+          <t>Callback URL</t>
+        </is>
+      </c>
+      <c r="D439" s="12" t="inlineStr">
+        <is>
+          <t>የመመለሻ አድራሻ</t>
+        </is>
+      </c>
+      <c r="E439" s="13" t="inlineStr">
+        <is>
+          <t>URL deebii</t>
+        </is>
+      </c>
+      <c r="F439" s="12" t="inlineStr">
+        <is>
+          <t>ኣድራሻ መመለሲ</t>
+        </is>
+      </c>
+      <c r="G439" s="13" t="inlineStr">
+        <is>
+          <t>URL-ka jawaabta</t>
+        </is>
+      </c>
+      <c r="H439" s="13" t="inlineStr">
+        <is>
+          <t>Kiungo cha kurudisha</t>
+        </is>
+      </c>
+      <c r="I439" s="14" t="inlineStr"/>
+    </row>
+    <row r="440" ht="44" customHeight="1">
+      <c r="A440" s="11" t="inlineStr">
+        <is>
+          <t>chan_verify_token</t>
+        </is>
+      </c>
+      <c r="B440" s="11" t="inlineStr">
+        <is>
+          <t>Read by bank staff, not customers. Keep it short — it has to fit the same space as the English. Use the words your branch staff already use.</t>
+        </is>
+      </c>
+      <c r="C440" s="11" t="inlineStr">
+        <is>
+          <t>Verify token</t>
+        </is>
+      </c>
+      <c r="D440" s="12" t="inlineStr">
+        <is>
+          <t>የማረጋገጫ ቶከን</t>
+        </is>
+      </c>
+      <c r="E440" s="13" t="inlineStr">
+        <is>
+          <t>Tokeenii mirkaneessaa</t>
+        </is>
+      </c>
+      <c r="F440" s="12" t="inlineStr">
+        <is>
+          <t>ቶከን መረጋገጺ</t>
+        </is>
+      </c>
+      <c r="G440" s="13" t="inlineStr">
+        <is>
+          <t>Token-ka xaqiijinta</t>
+        </is>
+      </c>
+      <c r="H440" s="13" t="inlineStr">
+        <is>
+          <t>Tokeni ya uthibitisho</t>
+        </is>
+      </c>
+      <c r="I440" s="14" t="inlineStr"/>
+    </row>
+    <row r="441" ht="44" customHeight="1">
+      <c r="A441" s="11" t="inlineStr">
+        <is>
+          <t>chan_meta_connected</t>
+        </is>
+      </c>
+      <c r="B441" s="11" t="inlineStr">
+        <is>
+          <t>Read by bank staff, not customers. Keep it short — it has to fit the same space as the English. Use the words your branch staff already use.</t>
+        </is>
+      </c>
+      <c r="C441" s="11" t="inlineStr">
+        <is>
+          <t>Meta credentials saved</t>
+        </is>
+      </c>
+      <c r="D441" s="12" t="inlineStr">
+        <is>
+          <t>የሜታ መረጃዎች ተቀምጠዋል</t>
+        </is>
+      </c>
+      <c r="E441" s="13" t="inlineStr">
+        <is>
+          <t>Ragaan Meta olkaa'ameera</t>
+        </is>
+      </c>
+      <c r="F441" s="12" t="inlineStr">
+        <is>
+          <t>ሓበሬታ ሜታ ተቐሚጡ</t>
+        </is>
+      </c>
+      <c r="G441" s="13" t="inlineStr">
+        <is>
+          <t>Aqoonsiga Meta waa la keydiyay</t>
+        </is>
+      </c>
+      <c r="H441" s="13" t="inlineStr">
+        <is>
+          <t>Vitambulisho vya Meta vimehifadhiwa</t>
+        </is>
+      </c>
+      <c r="I441" s="14" t="inlineStr"/>
+    </row>
+    <row r="442" ht="44" customHeight="1">
+      <c r="A442" s="11" t="inlineStr">
+        <is>
+          <t>chan_wa_phone_id</t>
+        </is>
+      </c>
+      <c r="B442" s="11" t="inlineStr">
+        <is>
+          <t>Read by bank staff, not customers. Keep it short — it has to fit the same space as the English. Use the words your branch staff already use.</t>
+        </is>
+      </c>
+      <c r="C442" s="11" t="inlineStr">
+        <is>
+          <t>WhatsApp phone number ID</t>
+        </is>
+      </c>
+      <c r="D442" s="12" t="inlineStr">
+        <is>
+          <t>የዋትስአፕ ስልክ ቁጥር መለያ</t>
+        </is>
+      </c>
+      <c r="E442" s="13" t="inlineStr">
+        <is>
+          <t>ID lakkoofsa bilbilaa WhatsApp</t>
+        </is>
+      </c>
+      <c r="F442" s="12" t="inlineStr">
+        <is>
+          <t>መለለዪ ቁጽሪ ተሌፎን ዋትስኣፕ</t>
+        </is>
+      </c>
+      <c r="G442" s="13" t="inlineStr">
+        <is>
+          <t>Aqoonsiga lambarka WhatsApp</t>
+        </is>
+      </c>
+      <c r="H442" s="13" t="inlineStr">
+        <is>
+          <t>Kitambulisho cha namba ya WhatsApp</t>
+        </is>
+      </c>
+      <c r="I442" s="14" t="inlineStr"/>
+    </row>
+    <row r="443" ht="44" customHeight="1">
+      <c r="A443" s="11" t="inlineStr">
+        <is>
+          <t>chan_wa_token</t>
+        </is>
+      </c>
+      <c r="B443" s="11" t="inlineStr">
+        <is>
+          <t>Read by bank staff, not customers. Keep it short — it has to fit the same space as the English. Use the words your branch staff already use.</t>
+        </is>
+      </c>
+      <c r="C443" s="11" t="inlineStr">
+        <is>
+          <t>WhatsApp access token</t>
+        </is>
+      </c>
+      <c r="D443" s="12" t="inlineStr">
+        <is>
+          <t>የዋትስአፕ መዳረሻ ቶከን</t>
+        </is>
+      </c>
+      <c r="E443" s="13" t="inlineStr">
+        <is>
+          <t>Tokeenii seensa WhatsApp</t>
+        </is>
+      </c>
+      <c r="F443" s="12" t="inlineStr">
+        <is>
+          <t>ቶከን መእተዊ ዋትስኣፕ</t>
+        </is>
+      </c>
+      <c r="G443" s="13" t="inlineStr">
+        <is>
+          <t>Token gelitaanka WhatsApp</t>
+        </is>
+      </c>
+      <c r="H443" s="13" t="inlineStr">
+        <is>
+          <t>Tokeni ya ufikiaji ya WhatsApp</t>
+        </is>
+      </c>
+      <c r="I443" s="14" t="inlineStr"/>
+    </row>
+    <row r="444" ht="44" customHeight="1">
+      <c r="A444" s="11" t="inlineStr">
+        <is>
+          <t>chan_ms_token</t>
+        </is>
+      </c>
+      <c r="B444" s="11" t="inlineStr">
+        <is>
+          <t>Read by bank staff, not customers. Keep it short — it has to fit the same space as the English. Use the words your branch staff already use.</t>
+        </is>
+      </c>
+      <c r="C444" s="11" t="inlineStr">
+        <is>
+          <t>Page access token</t>
+        </is>
+      </c>
+      <c r="D444" s="12" t="inlineStr">
+        <is>
+          <t>የገጽ መዳረሻ ቶከን</t>
+        </is>
+      </c>
+      <c r="E444" s="13" t="inlineStr">
+        <is>
+          <t>Tokeenii seensa fuulaa</t>
+        </is>
+      </c>
+      <c r="F444" s="12" t="inlineStr">
+        <is>
+          <t>ቶከን መእተዊ ገጽ</t>
+        </is>
+      </c>
+      <c r="G444" s="13" t="inlineStr">
+        <is>
+          <t>Token gelitaanka bogga</t>
+        </is>
+      </c>
+      <c r="H444" s="13" t="inlineStr">
+        <is>
+          <t>Tokeni ya ufikiaji ya ukurasa</t>
+        </is>
+      </c>
+      <c r="I444" s="14" t="inlineStr"/>
+    </row>
+    <row r="445" ht="44" customHeight="1">
+      <c r="A445" s="11" t="inlineStr">
+        <is>
+          <t>chan_ig_token</t>
+        </is>
+      </c>
+      <c r="B445" s="11" t="inlineStr">
+        <is>
+          <t>Read by bank staff, not customers. Keep it short — it has to fit the same space as the English. Use the words your branch staff already use.</t>
+        </is>
+      </c>
+      <c r="C445" s="11" t="inlineStr">
+        <is>
+          <t>Instagram access token</t>
+        </is>
+      </c>
+      <c r="D445" s="12" t="inlineStr">
+        <is>
+          <t>የኢንስታግራም መዳረሻ ቶከን</t>
+        </is>
+      </c>
+      <c r="E445" s="13" t="inlineStr">
+        <is>
+          <t>Tokeenii seensa Instagram</t>
+        </is>
+      </c>
+      <c r="F445" s="12" t="inlineStr">
+        <is>
+          <t>ቶከን መእተዊ ኢንስታግራም</t>
+        </is>
+      </c>
+      <c r="G445" s="13" t="inlineStr">
+        <is>
+          <t>Token gelitaanka Instagram</t>
+        </is>
+      </c>
+      <c r="H445" s="13" t="inlineStr">
+        <is>
+          <t>Tokeni ya ufikiaji ya Instagram</t>
+        </is>
+      </c>
+      <c r="I445" s="14" t="inlineStr"/>
+    </row>
+    <row r="446" ht="44" customHeight="1">
+      <c r="A446" s="11" t="inlineStr">
+        <is>
+          <t>chan_token_stored</t>
+        </is>
+      </c>
+      <c r="B446" s="11" t="inlineStr">
+        <is>
+          <t>Read by bank staff, not customers. Keep it short — it has to fit the same space as the English. Use the words your branch staff already use.</t>
+        </is>
+      </c>
+      <c r="C446" s="11" t="inlineStr">
+        <is>
+          <t>A token is already stored. Leave this blank to keep it.</t>
+        </is>
+      </c>
+      <c r="D446" s="12" t="inlineStr">
+        <is>
+          <t>ቶከን አስቀድሞ ተቀምጧል። ለማቆየት ይህን ባዶ ይተዉት።</t>
+        </is>
+      </c>
+      <c r="E446" s="13" t="inlineStr">
+        <is>
+          <t>Tokeeniin duraanuu olkaa'ameera. Isa tursiisuuf kana duwwaa dhiisaa.</t>
+        </is>
+      </c>
+      <c r="F446" s="12" t="inlineStr">
+        <is>
+          <t>ቶከን ድሮ ተቐሚጡ ኣሎ። ንምዕቃቡ ነዚ ባዶ ግደፍዎ።</t>
+        </is>
+      </c>
+      <c r="G446" s="13" t="inlineStr">
+        <is>
+          <t>Token horeyba waa la keydiyay. Si aad u hayso, banaan uga tag.</t>
+        </is>
+      </c>
+      <c r="H446" s="13" t="inlineStr">
+        <is>
+          <t>Tokeni tayari imehifadhiwa. Iache wazi ili kuiweka.</t>
+        </is>
+      </c>
+      <c r="I446" s="14" t="inlineStr"/>
+    </row>
+    <row r="447" ht="44" customHeight="1">
+      <c r="A447" s="11" t="inlineStr">
+        <is>
+          <t>chan_sms_title</t>
+        </is>
+      </c>
+      <c r="B447" s="11" t="inlineStr">
+        <is>
+          <t>Read by bank staff, not customers. Keep it short — it has to fit the same space as the English. Use the words your branch staff already use.</t>
+        </is>
+      </c>
+      <c r="C447" s="11" t="inlineStr">
+        <is>
+          <t>Connect your SMS gateway</t>
+        </is>
+      </c>
+      <c r="D447" s="12" t="inlineStr">
+        <is>
+          <t>የኤስኤምኤስ መተላለፊያዎን ያገናኙ</t>
+        </is>
+      </c>
+      <c r="E447" s="13" t="inlineStr">
+        <is>
+          <t>Karra SMS keessan wal qunnamsiisaa</t>
+        </is>
+      </c>
+      <c r="F447" s="12" t="inlineStr">
+        <is>
+          <t>መተሓላለፊ ኤስኤምኤስኩም ኣራኽቡ</t>
+        </is>
+      </c>
+      <c r="G447" s="13" t="inlineStr">
+        <is>
+          <t>Ku xidhiidhi albaabka SMS</t>
+        </is>
+      </c>
+      <c r="H447" s="13" t="inlineStr">
+        <is>
+          <t>Unganisha lango lako la SMS</t>
+        </is>
+      </c>
+      <c r="I447" s="14" t="inlineStr"/>
+    </row>
+    <row r="448" ht="44" customHeight="1">
+      <c r="A448" s="11" t="inlineStr">
+        <is>
+          <t>chan_sms_help</t>
+        </is>
+      </c>
+      <c r="B448" s="11" t="inlineStr">
+        <is>
+          <t>Read by bank staff, not customers. Keep it short — it has to fit the same space as the English. Use the words your branch staff already use.</t>
+        </is>
+      </c>
+      <c r="C448" s="11" t="inlineStr">
+        <is>
+          <t>SMS is the one channel with no single vendor API, so this takes your aggregator's own send URL. Every reply on this channel costs money.</t>
+        </is>
+      </c>
+      <c r="D448" s="12" t="inlineStr">
+        <is>
+          <t>ኤስኤምኤስ አንድ የጋራ የአቅራቢ ኤፒአይ የሌለው ብቸኛው መስመር ነው፤ ስለዚህ የአቅራቢዎን የመላኪያ አድራሻ ይፈልጋል። በዚህ መስመር ላይ እያንዳንዱ ምላሽ ገንዘብ ያስወጣል።</t>
+        </is>
+      </c>
+      <c r="E448" s="13" t="inlineStr">
+        <is>
+          <t>SMS karaa API dhiyeessaa tokkichi hin jirre qofa, kanaafuu URL ergaa dhiyeessaa keessanii barbaada. Karaa kanarratti deebiin hundi baasii qaba.</t>
+        </is>
+      </c>
+      <c r="F448" s="12" t="inlineStr">
+        <is>
+          <t>ኤስኤምኤስ ሓደ ንኹሉ ዝኸውን ኤፒኣይ ዘይብሉ እንኮ መስመር እዩ፣ ስለዚ ናይ ኣቕራቢኹም ኣድራሻ መስደዲ የድሊ። ኣብዚ መስመር ነፍሲ ወከፍ መልሲ ገንዘብ የውጽእ።</t>
+        </is>
+      </c>
+      <c r="G448" s="13" t="inlineStr">
+        <is>
+          <t>SMS waa kanaalka kaliya ee aan lahayn hal API oo iibiye, sidaas darteed wuxuu u baahan yahay URL-ka dirista ee shirkaddaada. Kanaalkan jawaab kastaa lacag bay ku baxdaa.</t>
+        </is>
+      </c>
+      <c r="H448" s="13" t="inlineStr">
+        <is>
+          <t>SMS ndiyo njia pekee isiyo na API moja ya muuzaji, kwa hivyo inahitaji kiungo cha kutuma cha mtoa huduma wako. Kila jibu kwenye njia hii lina gharama.</t>
+        </is>
+      </c>
+      <c r="I448" s="14" t="inlineStr"/>
+    </row>
+    <row r="449" ht="44" customHeight="1">
+      <c r="A449" s="11" t="inlineStr">
+        <is>
+          <t>chan_sms_url</t>
+        </is>
+      </c>
+      <c r="B449" s="11" t="inlineStr">
+        <is>
+          <t>Read by bank staff, not customers. Keep it short — it has to fit the same space as the English. Use the words your branch staff already use.</t>
+        </is>
+      </c>
+      <c r="C449" s="11" t="inlineStr">
+        <is>
+          <t>Send URL</t>
+        </is>
+      </c>
+      <c r="D449" s="12" t="inlineStr">
+        <is>
+          <t>የመላኪያ አድራሻ</t>
+        </is>
+      </c>
+      <c r="E449" s="13" t="inlineStr">
+        <is>
+          <t>URL ergaa</t>
+        </is>
+      </c>
+      <c r="F449" s="12" t="inlineStr">
+        <is>
+          <t>ኣድራሻ መስደዲ</t>
+        </is>
+      </c>
+      <c r="G449" s="13" t="inlineStr">
+        <is>
+          <t>URL-ka dirista</t>
+        </is>
+      </c>
+      <c r="H449" s="13" t="inlineStr">
+        <is>
+          <t>Kiungo cha kutuma</t>
+        </is>
+      </c>
+      <c r="I449" s="14" t="inlineStr"/>
+    </row>
+    <row r="450" ht="44" customHeight="1">
+      <c r="A450" s="11" t="inlineStr">
+        <is>
+          <t>chan_sms_auth</t>
+        </is>
+      </c>
+      <c r="B450" s="11" t="inlineStr">
+        <is>
+          <t>Read by bank staff, not customers. Keep it short — it has to fit the same space as the English. Use the words your branch staff already use.</t>
+        </is>
+      </c>
+      <c r="C450" s="11" t="inlineStr">
+        <is>
+          <t>Authorization header</t>
+        </is>
+      </c>
+      <c r="D450" s="12" t="inlineStr">
+        <is>
+          <t>የፈቃድ ራስጌ</t>
+        </is>
+      </c>
+      <c r="E450" s="13" t="inlineStr">
+        <is>
+          <t>Mataduree hayyamaa</t>
+        </is>
+      </c>
+      <c r="F450" s="12" t="inlineStr">
+        <is>
+          <t>ርእሲ ፍቓድ</t>
+        </is>
+      </c>
+      <c r="G450" s="13" t="inlineStr">
+        <is>
+          <t>Madaxa oggolaanshaha</t>
+        </is>
+      </c>
+      <c r="H450" s="13" t="inlineStr">
+        <is>
+          <t>Kichwa cha idhini</t>
+        </is>
+      </c>
+      <c r="I450" s="14" t="inlineStr"/>
+    </row>
+    <row r="451" ht="44" customHeight="1">
+      <c r="A451" s="11" t="inlineStr">
+        <is>
+          <t>chan_sms_auth_help</t>
+        </is>
+      </c>
+      <c r="B451" s="11" t="inlineStr">
+        <is>
+          <t>Read by bank staff, not customers. Keep it short — it has to fit the same space as the English. Use the words your branch staff already use.</t>
+        </is>
+      </c>
+      <c r="C451" s="11" t="inlineStr">
+        <is>
+          <t>Sent with every outbound message — usually Bearer or Basic, exactly as your aggregator documents it.</t>
+        </is>
+      </c>
+      <c r="D451" s="12" t="inlineStr">
+        <is>
+          <t>ከእያንዳንዱ ወጪ መልእክት ጋር ይላካል — ብዙውን ጊዜ Bearer ወይም Basic፣ አቅራቢዎ በሚገልጸው መልኩ በትክክል።</t>
+        </is>
+      </c>
+      <c r="E451" s="13" t="inlineStr">
+        <is>
+          <t>Ergaa ba'u hunda waliin ergama — yeroo baay'ee Bearer yookaan Basic, akkuma dhiyeessaan keessan barreesse.</t>
+        </is>
+      </c>
+      <c r="F451" s="12" t="inlineStr">
+        <is>
+          <t>ምስ ነፍሲ ወከፍ ወጻኢ መልእኽቲ ይስደድ — መብዛሕትኡ ግዜ Bearer ወይ Basic፣ ልክዕ ከምቲ ኣቕራቢኹም ዝገልጾ።</t>
+        </is>
+      </c>
+      <c r="G451" s="13" t="inlineStr">
+        <is>
+          <t>Waxaa la diraa fariin kasta oo baxaysa — badanaa Bearer ama Basic, sida uu shirkaddaadu u qoray.</t>
+        </is>
+      </c>
+      <c r="H451" s="13" t="inlineStr">
+        <is>
+          <t>Hutumwa na kila ujumbe unaotoka — kwa kawaida Bearer au Basic, hasa kama mtoa huduma wako anavyoeleza.</t>
+        </is>
+      </c>
+      <c r="I451" s="14" t="inlineStr"/>
+    </row>
+    <row r="452" ht="44" customHeight="1">
+      <c r="A452" s="11" t="inlineStr">
+        <is>
+          <t>chan_sms_auth_stored</t>
+        </is>
+      </c>
+      <c r="B452" s="11" t="inlineStr">
+        <is>
+          <t>Read by bank staff, not customers. Keep it short — it has to fit the same space as the English. Use the words your branch staff already use.</t>
+        </is>
+      </c>
+      <c r="C452" s="11" t="inlineStr">
+        <is>
+          <t>An authorization header is stored. Leave this blank to keep it.</t>
+        </is>
+      </c>
+      <c r="D452" s="12" t="inlineStr">
+        <is>
+          <t>የፈቃድ ራስጌ ተቀምጧል። ለማቆየት ይህን ባዶ ይተዉት።</t>
+        </is>
+      </c>
+      <c r="E452" s="13" t="inlineStr">
+        <is>
+          <t>Mataduree hayyamaa olkaa'ameera. Isa tursiisuuf kana duwwaa dhiisaa.</t>
+        </is>
+      </c>
+      <c r="F452" s="12" t="inlineStr">
+        <is>
+          <t>ርእሲ ፍቓድ ተቐሚጡ ኣሎ። ንምዕቃቡ ነዚ ባዶ ግደፍዎ።</t>
+        </is>
+      </c>
+      <c r="G452" s="13" t="inlineStr">
+        <is>
+          <t>Madax oggolaansho ah waa la keydiyay. Si aad u hayso, banaan uga tag.</t>
+        </is>
+      </c>
+      <c r="H452" s="13" t="inlineStr">
+        <is>
+          <t>Kichwa cha idhini kimehifadhiwa. Kiache wazi ili kukiweka.</t>
+        </is>
+      </c>
+      <c r="I452" s="14" t="inlineStr"/>
+    </row>
+    <row r="453" ht="44" customHeight="1">
+      <c r="A453" s="11" t="inlineStr">
+        <is>
+          <t>chan_sms_sender</t>
+        </is>
+      </c>
+      <c r="B453" s="11" t="inlineStr">
+        <is>
+          <t>Read by bank staff, not customers. Keep it short — it has to fit the same space as the English. Use the words your branch staff already use.</t>
+        </is>
+      </c>
+      <c r="C453" s="11" t="inlineStr">
+        <is>
+          <t>Sender ID or shortcode</t>
+        </is>
+      </c>
+      <c r="D453" s="12" t="inlineStr">
+        <is>
+          <t>የላኪ መለያ ወይም አጭር ቁጥር</t>
+        </is>
+      </c>
+      <c r="E453" s="13" t="inlineStr">
+        <is>
+          <t>ID ergaa yookaan lakkoofsa gabaabaa</t>
+        </is>
+      </c>
+      <c r="F453" s="12" t="inlineStr">
+        <is>
+          <t>መለለዪ ሰዳዲ ወይ ሓጺር ቁጽሪ</t>
+        </is>
+      </c>
+      <c r="G453" s="13" t="inlineStr">
+        <is>
+          <t>Aqoonsiga diraha ama lambar gaaban</t>
+        </is>
+      </c>
+      <c r="H453" s="13" t="inlineStr">
+        <is>
+          <t>Kitambulisho cha mtumaji au namba fupi</t>
+        </is>
+      </c>
+      <c r="I453" s="14" t="inlineStr"/>
+    </row>
+    <row r="454" ht="44" customHeight="1">
+      <c r="A454" s="11" t="inlineStr">
+        <is>
+          <t>chan_sms_inbound_title</t>
+        </is>
+      </c>
+      <c r="B454" s="11" t="inlineStr">
+        <is>
+          <t>Read by bank staff, not customers. Keep it short — it has to fit the same space as the English. Use the words your branch staff already use.</t>
+        </is>
+      </c>
+      <c r="C454" s="11" t="inlineStr">
+        <is>
+          <t>Point your aggregator here</t>
+        </is>
+      </c>
+      <c r="D454" s="12" t="inlineStr">
+        <is>
+          <t>አቅራቢዎን ወደዚህ ያመልክቱ</t>
+        </is>
+      </c>
+      <c r="E454" s="13" t="inlineStr">
+        <is>
+          <t>Dhiyeessaa keessan gara kanaatti qajeelchaa</t>
+        </is>
+      </c>
+      <c r="F454" s="12" t="inlineStr">
+        <is>
+          <t>ንኣቕራቢኹም ናብዚ ኣመልክቱ</t>
+        </is>
+      </c>
+      <c r="G454" s="13" t="inlineStr">
+        <is>
+          <t>Shirkaddaada halkan u tilmaan</t>
+        </is>
+      </c>
+      <c r="H454" s="13" t="inlineStr">
+        <is>
+          <t>Elekeza mtoa huduma wako hapa</t>
+        </is>
+      </c>
+      <c r="I454" s="14" t="inlineStr"/>
+    </row>
+    <row r="455" ht="44" customHeight="1">
+      <c r="A455" s="11" t="inlineStr">
+        <is>
+          <t>chan_sms_inbound_help</t>
+        </is>
+      </c>
+      <c r="B455" s="11" t="inlineStr">
+        <is>
+          <t>Read by bank staff, not customers. Keep it short — it has to fit the same space as the English. Use the words your branch staff already use.</t>
+        </is>
+      </c>
+      <c r="C455" s="11" t="inlineStr">
+        <is>
+          <t>Give your aggregator this URL for inbound messages, and have it send the secret below as an X-SMS-Secret header. Without a matching secret every inbound message is refused.</t>
+        </is>
+      </c>
+      <c r="D455" s="12" t="inlineStr">
+        <is>
+          <t>ለገቢ መልእክቶች ይህን አድራሻ ለአቅራቢዎ ይስጡ፤ ከታች ያለውን ሚስጥር እንደ X-SMS-Secret ራስጌ እንዲልክ ያድርጉ። የሚዛመድ ሚስጥር ከሌለ እያንዳንዱ ገቢ መልእክት ይከለከላል።</t>
+        </is>
+      </c>
+      <c r="E455" s="13" t="inlineStr">
+        <is>
+          <t>Ergaawwan seenaniif URL kana dhiyeessaa keessaniif kennaa, iccitii armaan gadii akka mataduree X-SMS-Secret akka ergu godhaa. Iccitii wal simu malee ergaan seenu hundi ni dhorkama.</t>
+        </is>
+      </c>
+      <c r="F455" s="12" t="inlineStr">
+        <is>
+          <t>ንዝኣትዉ መልእኽትታት ነዚ ኣድራሻ ንኣቕራቢኹም ሃብዎ፣ ነቲ ኣብ ታሕቲ ዘሎ ምስጢር ከም ርእሲ X-SMS-Secret ክሰድዶ ግበሩ። ዝሰማማዕ ምስጢር እንተዘየልዩ ነፍሲ ወከፍ ዝኣቱ መልእኽቲ ይእገድ።</t>
+        </is>
+      </c>
+      <c r="G455" s="13" t="inlineStr">
+        <is>
+          <t>Shirkaddaada sii URL-kan fariimaha soo gelaya, oo ka dhig inay sirta hoose u soo dirto sida madax X-SMS-Secret ah. Sir is-waafaqsan la'aanteed fariin kasta oo soo gelaysa waa la diidayaa.</t>
+        </is>
+      </c>
+      <c r="H455" s="13" t="inlineStr">
+        <is>
+          <t>Mpe mtoa huduma wako kiungo hiki kwa ujumbe unaoingia, na ufanye atume siri iliyo hapa chini kama kichwa cha X-SMS-Secret. Bila siri inayolingana kila ujumbe unaoingia unakataliwa.</t>
+        </is>
+      </c>
+      <c r="I455" s="14" t="inlineStr"/>
+    </row>
+    <row r="456" ht="44" customHeight="1">
+      <c r="A456" s="11" t="inlineStr">
+        <is>
+          <t>chan_sms_secret_once</t>
+        </is>
+      </c>
+      <c r="B456" s="11" t="inlineStr">
+        <is>
+          <t>Read by bank staff, not customers. Keep it short — it has to fit the same space as the English. Use the words your branch staff already use.</t>
+        </is>
+      </c>
+      <c r="C456" s="11" t="inlineStr">
+        <is>
+          <t>Copy this now — it is shown once and never again.</t>
+        </is>
+      </c>
+      <c r="D456" s="12" t="inlineStr">
+        <is>
+          <t>አሁን ይቅዱት — አንድ ጊዜ ብቻ ይታያል፤ እንደገና አይታይም።</t>
+        </is>
+      </c>
+      <c r="E456" s="13" t="inlineStr">
+        <is>
+          <t>Amma garagalchaa — yeroo tokko qofa mul'ata, lammata hin mul'atu.</t>
+        </is>
+      </c>
+      <c r="F456" s="12" t="inlineStr">
+        <is>
+          <t>ሕጂ ቅድሕዎ — ሓንሳብ ጥራይ እዩ ዝርአ፣ ደጊሙ ኣይርአን።</t>
+        </is>
+      </c>
+      <c r="G456" s="13" t="inlineStr">
+        <is>
+          <t>Hadda koobiyee — hal mar ayaa la tusayaa, marnaba mar labaad lama tusayo.</t>
+        </is>
+      </c>
+      <c r="H456" s="13" t="inlineStr">
+        <is>
+          <t>Nakili sasa — inaonyeshwa mara moja tu na kamwe tena.</t>
+        </is>
+      </c>
+      <c r="I456" s="14" t="inlineStr"/>
+    </row>
+    <row r="457" ht="44" customHeight="1">
+      <c r="A457" s="11" t="inlineStr">
+        <is>
+          <t>chan_sms_secret_set</t>
+        </is>
+      </c>
+      <c r="B457" s="11" t="inlineStr">
+        <is>
+          <t>Read by bank staff, not customers. Keep it short — it has to fit the same space as the English. Use the words your branch staff already use.</t>
+        </is>
+      </c>
+      <c r="C457" s="11" t="inlineStr">
+        <is>
+          <t>An inbound secret is set. It is shown only when first created — reconnecting keeps the same one.</t>
+        </is>
+      </c>
+      <c r="D457" s="12" t="inlineStr">
+        <is>
+          <t>የገቢ ሚስጥር ተዘጋጅቷል። ሲፈጠር ብቻ ነው የሚታየው — እንደገና ማገናኘት ተመሳሳዩን ያቆያል።</t>
+        </is>
+      </c>
+      <c r="E457" s="13" t="inlineStr">
+        <is>
+          <t>Iccitiin seensaa qophaa'eera. Yeroo jalqabaa uumamu qofa mul'ata — irra deebi'anii wal qunnamsiisuun isuma tursiisa.</t>
+        </is>
+      </c>
+      <c r="F457" s="12" t="inlineStr">
+        <is>
+          <t>ምስጢር መእተዊ ተቐሚጡ ኣሎ። ኣብ መጀመርታ ክፍጠር ከሎ ጥራይ እዩ ዝርአ — መሊስካ ምርኻብ ነቲ ሓደ የቐምጦ።</t>
+        </is>
+      </c>
+      <c r="G457" s="13" t="inlineStr">
+        <is>
+          <t>Sir gelitaan ah waa la dejiyay. Waxaa la tusaa markii ugu horreysay ee la abuuro oo kaliya — dib u xidhiidhinta isla midkaas ayay haysaa.</t>
+        </is>
+      </c>
+      <c r="H457" s="13" t="inlineStr">
+        <is>
+          <t>Siri ya ujumbe unaoingia imewekwa. Inaonyeshwa tu inapoundwa mara ya kwanza — kuunganisha upya kunahifadhi ile ile.</t>
+        </is>
+      </c>
+      <c r="I457" s="14" t="inlineStr"/>
+    </row>
+    <row r="458" ht="44" customHeight="1">
+      <c r="A458" s="11" t="inlineStr">
+        <is>
+          <t>chan_sms_connected</t>
+        </is>
+      </c>
+      <c r="B458" s="11" t="inlineStr">
+        <is>
+          <t>Read by bank staff, not customers. Keep it short — it has to fit the same space as the English. Use the words your branch staff already use.</t>
+        </is>
+      </c>
+      <c r="C458" s="11" t="inlineStr">
+        <is>
+          <t>SMS gateway connected</t>
+        </is>
+      </c>
+      <c r="D458" s="12" t="inlineStr">
+        <is>
+          <t>የኤስኤምኤስ መተላለፊያ ተገናኝቷል</t>
+        </is>
+      </c>
+      <c r="E458" s="13" t="inlineStr">
+        <is>
+          <t>Karri SMS wal qunnameera</t>
+        </is>
+      </c>
+      <c r="F458" s="12" t="inlineStr">
+        <is>
+          <t>መተሓላለፊ ኤስኤምኤስ ተራኺቡ</t>
+        </is>
+      </c>
+      <c r="G458" s="13" t="inlineStr">
+        <is>
+          <t>Albaabka SMS waa la xidhiidhiyay</t>
+        </is>
+      </c>
+      <c r="H458" s="13" t="inlineStr">
+        <is>
+          <t>Lango la SMS limeunganishwa</t>
+        </is>
+      </c>
+      <c r="I458" s="14" t="inlineStr"/>
+    </row>
+    <row r="459" ht="44" customHeight="1">
+      <c r="A459" s="11" t="inlineStr">
+        <is>
+          <t>chan_sms_secret_label</t>
+        </is>
+      </c>
+      <c r="B459" s="11" t="inlineStr">
+        <is>
+          <t>Read by bank staff, not customers. Keep it short — it has to fit the same space as the English. Use the words your branch staff already use.</t>
+        </is>
+      </c>
+      <c r="C459" s="11" t="inlineStr">
+        <is>
+          <t>Inbound secret</t>
+        </is>
+      </c>
+      <c r="D459" s="12" t="inlineStr">
+        <is>
+          <t>የገቢ ሚስጥር</t>
+        </is>
+      </c>
+      <c r="E459" s="13" t="inlineStr">
+        <is>
+          <t>Iccitii seensaa</t>
+        </is>
+      </c>
+      <c r="F459" s="12" t="inlineStr">
+        <is>
+          <t>ምስጢር መእተዊ</t>
+        </is>
+      </c>
+      <c r="G459" s="13" t="inlineStr">
+        <is>
+          <t>Sirta gelitaanka</t>
+        </is>
+      </c>
+      <c r="H459" s="13" t="inlineStr">
+        <is>
+          <t>Siri ya ujumbe unaoingia</t>
+        </is>
+      </c>
+      <c r="I459" s="14" t="inlineStr"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:I417"/>
+  <autoFilter ref="A1:I459"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
feat: a fresh tenant is told what to do first (#176)
A new tenant's dashboard was honest and useless: every number zeroed and
nowhere the one fact that mattered — no knowledge base, so the assistant
can answer nothing.

GET /admin/api/{slug}/setup reports readiness and the dashboard renders
it first on the page. Staged by data rather than date, read all-time so a
quiet month never resurrects it, and retired by the first real customer
conversation — preview traffic cannot retire it (ADR-0036). Shown only to
someone who can act on it.

Also fixes the conversations-per-day chart, whose empty state never fired
because the backend fills the window: thirty zero-count days passed a
length check and drew a void.

Thirteen strings in six languages; workbook regenerated. New bare_bank
fixture — no fixture had ever rendered the product empty.
</commit_message>
<xml_diff>
--- a/review/Olink_Bank_Assist_language_review.xlsx
+++ b/review/Olink_Bank_Assist_language_review.xlsx
@@ -17,7 +17,7 @@
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'1. What the assistant says'!$A$1:$I$24</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'2. What it understands'!$A$1:$E$91</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'3. Buttons customers see'!$A$1:$I$53</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'4. The staff panel'!$A$1:$I$459</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'4. The staff panel'!$A$1:$I$472</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -752,7 +752,7 @@
       </c>
       <c r="C26" s="6" t="inlineStr">
         <is>
-          <t>533 strings in 5 languages</t>
+          <t>546 strings in 5 languages</t>
         </is>
       </c>
     </row>
@@ -6345,7 +6345,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I459"/>
+  <dimension ref="A1:I472"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
@@ -26100,8 +26100,567 @@
       </c>
       <c r="I459" s="14" t="inlineStr"/>
     </row>
+    <row r="460" ht="44" customHeight="1">
+      <c r="A460" s="11" t="inlineStr">
+        <is>
+          <t>setup_title</t>
+        </is>
+      </c>
+      <c r="B460" s="11" t="inlineStr">
+        <is>
+          <t>Read by bank staff, not customers. Keep it short — it has to fit the same space as the English. Use the words your branch staff already use.</t>
+        </is>
+      </c>
+      <c r="C460" s="11" t="inlineStr">
+        <is>
+          <t>Get your assistant ready</t>
+        </is>
+      </c>
+      <c r="D460" s="12" t="inlineStr">
+        <is>
+          <t>ረዳትዎን ያዘጋጁ</t>
+        </is>
+      </c>
+      <c r="E460" s="13" t="inlineStr">
+        <is>
+          <t>Gargaaraa kee qopheessi</t>
+        </is>
+      </c>
+      <c r="F460" s="12" t="inlineStr">
+        <is>
+          <t>ንሓጋዚኻ ኣዳልዎ</t>
+        </is>
+      </c>
+      <c r="G460" s="13" t="inlineStr">
+        <is>
+          <t>Kaaliyahaaga diyaari</t>
+        </is>
+      </c>
+      <c r="H460" s="13" t="inlineStr">
+        <is>
+          <t>Andaa msaidizi wako</t>
+        </is>
+      </c>
+      <c r="I460" s="14" t="inlineStr"/>
+    </row>
+    <row r="461" ht="44" customHeight="1">
+      <c r="A461" s="11" t="inlineStr">
+        <is>
+          <t>setup_sub</t>
+        </is>
+      </c>
+      <c r="B461" s="11" t="inlineStr">
+        <is>
+          <t>Read by bank staff, not customers. Keep it short — it has to fit the same space as the English. Use the words your branch staff already use.</t>
+        </is>
+      </c>
+      <c r="C461" s="11" t="inlineStr">
+        <is>
+          <t>A few things to set up before your customers arrive. This disappears once the first customer writes in.</t>
+        </is>
+      </c>
+      <c r="D461" s="12" t="inlineStr">
+        <is>
+          <t>ደንበኞችዎ ከመምጣታቸው በፊት የሚዘጋጁ ጥቂት ነገሮች። የመጀመሪያው ደንበኛ እንደጻፈ ይህ ይጠፋል።</t>
+        </is>
+      </c>
+      <c r="E461" s="13" t="inlineStr">
+        <is>
+          <t>Maamiltoonni kee dura wantoota muraasa qopheessuu qabdu. Maamilaan jalqabaa yeroo barreessu kun ni bada.</t>
+        </is>
+      </c>
+      <c r="F461" s="12" t="inlineStr">
+        <is>
+          <t>ዓማዊልካ ቅድሚ ምምጻኦም ዘዳልዉ ቁሩብ ነገራት። እቲ ቀዳማይ ዓሚል ምስ ጸሓፈ እዚ ይጠፍእ።</t>
+        </is>
+      </c>
+      <c r="G461" s="13" t="inlineStr">
+        <is>
+          <t>Dhowr shay oo aad diyaarin lahayd ka hor inta aan macaamiishaadu iman. Tani way baaba'daa marka macmiilka koowaad qoro.</t>
+        </is>
+      </c>
+      <c r="H461" s="13" t="inlineStr">
+        <is>
+          <t>Mambo machache ya kuandaa kabla wateja wako hawajafika. Hii hupotea mteja wa kwanza anapoandika.</t>
+        </is>
+      </c>
+      <c r="I461" s="14" t="inlineStr"/>
+    </row>
+    <row r="462" ht="44" customHeight="1">
+      <c r="A462" s="11" t="inlineStr">
+        <is>
+          <t>setup_progress</t>
+        </is>
+      </c>
+      <c r="B462" s="11" t="inlineStr">
+        <is>
+          <t>Read by bank staff, not customers. Keep it short — it has to fit the same space as the English. Use the words your branch staff already use.</t>
+        </is>
+      </c>
+      <c r="C462" s="11" t="inlineStr">
+        <is>
+          <t>{done} of {total} done</t>
+        </is>
+      </c>
+      <c r="D462" s="12" t="inlineStr">
+        <is>
+          <t>ከ{total} {done} ተጠናቅቋል</t>
+        </is>
+      </c>
+      <c r="E462" s="13" t="inlineStr">
+        <is>
+          <t>{total} keessaa {done} xumurameera</t>
+        </is>
+      </c>
+      <c r="F462" s="12" t="inlineStr">
+        <is>
+          <t>ካብ {total} {done} ተወዲኡ</t>
+        </is>
+      </c>
+      <c r="G462" s="13" t="inlineStr">
+        <is>
+          <t>{done} ka mid ah {total} ayaa dhammaaday</t>
+        </is>
+      </c>
+      <c r="H462" s="13" t="inlineStr">
+        <is>
+          <t>{done} kati ya {total} yamekamilika</t>
+        </is>
+      </c>
+      <c r="I462" s="14" t="inlineStr"/>
+    </row>
+    <row r="463" ht="44" customHeight="1">
+      <c r="A463" s="11" t="inlineStr">
+        <is>
+          <t>setup_knowledge</t>
+        </is>
+      </c>
+      <c r="B463" s="11" t="inlineStr">
+        <is>
+          <t>Read by bank staff, not customers. Keep it short — it has to fit the same space as the English. Use the words your branch staff already use.</t>
+        </is>
+      </c>
+      <c r="C463" s="11" t="inlineStr">
+        <is>
+          <t>Add your knowledge base</t>
+        </is>
+      </c>
+      <c r="D463" s="12" t="inlineStr">
+        <is>
+          <t>የእውቀት ማከማቻዎን ያስገቡ</t>
+        </is>
+      </c>
+      <c r="E463" s="13" t="inlineStr">
+        <is>
+          <t>Kuusaa beekumsa kee galchi</t>
+        </is>
+      </c>
+      <c r="F463" s="12" t="inlineStr">
+        <is>
+          <t>ናይ ፍልጠት መኽዘንካ ኣእቱ</t>
+        </is>
+      </c>
+      <c r="G463" s="13" t="inlineStr">
+        <is>
+          <t>Kuur aqooneed kaaga dar</t>
+        </is>
+      </c>
+      <c r="H463" s="13" t="inlineStr">
+        <is>
+          <t>Ongeza hifadhi yako ya maarifa</t>
+        </is>
+      </c>
+      <c r="I463" s="14" t="inlineStr"/>
+    </row>
+    <row r="464" ht="44" customHeight="1">
+      <c r="A464" s="11" t="inlineStr">
+        <is>
+          <t>setup_knowledge_help</t>
+        </is>
+      </c>
+      <c r="B464" s="11" t="inlineStr">
+        <is>
+          <t>Read by bank staff, not customers. Keep it short — it has to fit the same space as the English. Use the words your branch staff already use.</t>
+        </is>
+      </c>
+      <c r="C464" s="11" t="inlineStr">
+        <is>
+          <t>Until this has content the assistant can answer nothing — it will hand every question to a person.</t>
+        </is>
+      </c>
+      <c r="D464" s="12" t="inlineStr">
+        <is>
+          <t>ይህ ይዘት እስከሌለው ድረስ ረዳቱ ምንም መመለስ አይችልም — እያንዳንዱን ጥያቄ ወደ ሰው ያስተላልፋል።</t>
+        </is>
+      </c>
+      <c r="E464" s="13" t="inlineStr">
+        <is>
+          <t>Hanga kun qabiyyee qabaatutti gargaaraan homaa deebisuu hin danda'u — gaaffii hunda nama biratti dabarsa.</t>
+        </is>
+      </c>
+      <c r="F464" s="12" t="inlineStr">
+        <is>
+          <t>እዚ ትሕዝቶ ክሳብ ዘይብሉ ሓጋዚ ገለ ክምልስ ኣይክእልን — ንኹሉ ሕቶ ናብ ሰብ የመሓላልፎ።</t>
+        </is>
+      </c>
+      <c r="G464" s="13" t="inlineStr">
+        <is>
+          <t>Ilaa tani ay waxyaabo yeelato kaaliyuhu waxba ma jawaabi karo — su'aal walba wuxuu u gudbin doonaa qof.</t>
+        </is>
+      </c>
+      <c r="H464" s="13" t="inlineStr">
+        <is>
+          <t>Hadi hii iwe na maudhui msaidizi hawezi kujibu chochote — atapeleka kila swali kwa mtu.</t>
+        </is>
+      </c>
+      <c r="I464" s="14" t="inlineStr"/>
+    </row>
+    <row r="465" ht="44" customHeight="1">
+      <c r="A465" s="11" t="inlineStr">
+        <is>
+          <t>setup_brand</t>
+        </is>
+      </c>
+      <c r="B465" s="11" t="inlineStr">
+        <is>
+          <t>Read by bank staff, not customers. Keep it short — it has to fit the same space as the English. Use the words your branch staff already use.</t>
+        </is>
+      </c>
+      <c r="C465" s="11" t="inlineStr">
+        <is>
+          <t>Make it look like your bank</t>
+        </is>
+      </c>
+      <c r="D465" s="12" t="inlineStr">
+        <is>
+          <t>የባንክዎን መልክ ይስጡት</t>
+        </is>
+      </c>
+      <c r="E465" s="13" t="inlineStr">
+        <is>
+          <t>Bifa baankii keetii itti kenni</t>
+        </is>
+      </c>
+      <c r="F465" s="12" t="inlineStr">
+        <is>
+          <t>ናይ ባንክኻ መልክዕ ሃቦ</t>
+        </is>
+      </c>
+      <c r="G465" s="13" t="inlineStr">
+        <is>
+          <t>Muuqaal bankigaaga u yeel</t>
+        </is>
+      </c>
+      <c r="H465" s="13" t="inlineStr">
+        <is>
+          <t>Ipe sura ya benki yako</t>
+        </is>
+      </c>
+      <c r="I465" s="14" t="inlineStr"/>
+    </row>
+    <row r="466" ht="44" customHeight="1">
+      <c r="A466" s="11" t="inlineStr">
+        <is>
+          <t>setup_brand_help</t>
+        </is>
+      </c>
+      <c r="B466" s="11" t="inlineStr">
+        <is>
+          <t>Read by bank staff, not customers. Keep it short — it has to fit the same space as the English. Use the words your branch staff already use.</t>
+        </is>
+      </c>
+      <c r="C466" s="11" t="inlineStr">
+        <is>
+          <t>Your colour and logo, so a customer recognises the assistant as yours.</t>
+        </is>
+      </c>
+      <c r="D466" s="12" t="inlineStr">
+        <is>
+          <t>ቀለምዎና አርማዎ፣ ደንበኛ ረዳቱን የእርስዎ መሆኑን እንዲያውቅ።</t>
+        </is>
+      </c>
+      <c r="E466" s="13" t="inlineStr">
+        <is>
+          <t>Halluu fi asxaa kee, akka maamilaan gargaaraan kan kee ta'uu beekuuf.</t>
+        </is>
+      </c>
+      <c r="F466" s="12" t="inlineStr">
+        <is>
+          <t>ሕብርኻን ኣርማኻን፡ ዓሚል ነቲ ሓጋዚ ናትካ ምዃኑ ምእንቲ ክፈልጦ።</t>
+        </is>
+      </c>
+      <c r="G466" s="13" t="inlineStr">
+        <is>
+          <t>Midabkaaga iyo astaantaada, si macmiilku u garto kaaliyuhu inuu kaaga yahay.</t>
+        </is>
+      </c>
+      <c r="H466" s="13" t="inlineStr">
+        <is>
+          <t>Rangi na nembo yako, ili mteja atambue msaidizi kuwa ni wako.</t>
+        </is>
+      </c>
+      <c r="I466" s="14" t="inlineStr"/>
+    </row>
+    <row r="467" ht="44" customHeight="1">
+      <c r="A467" s="11" t="inlineStr">
+        <is>
+          <t>setup_channels</t>
+        </is>
+      </c>
+      <c r="B467" s="11" t="inlineStr">
+        <is>
+          <t>Read by bank staff, not customers. Keep it short — it has to fit the same space as the English. Use the words your branch staff already use.</t>
+        </is>
+      </c>
+      <c r="C467" s="11" t="inlineStr">
+        <is>
+          <t>Reach customers where they already are</t>
+        </is>
+      </c>
+      <c r="D467" s="12" t="inlineStr">
+        <is>
+          <t>ደንበኞችን ባሉበት ይድረሱ</t>
+        </is>
+      </c>
+      <c r="E467" s="13" t="inlineStr">
+        <is>
+          <t>Maamiltoota bakka jiranitti dhaqqabi</t>
+        </is>
+      </c>
+      <c r="F467" s="12" t="inlineStr">
+        <is>
+          <t>ንዓማዊል ኣብ ዘለውዎ በጽሓዮም</t>
+        </is>
+      </c>
+      <c r="G467" s="13" t="inlineStr">
+        <is>
+          <t>Macaamiisha gaadh meesha ay hore ugu joogaan</t>
+        </is>
+      </c>
+      <c r="H467" s="13" t="inlineStr">
+        <is>
+          <t>Wafikie wateja walipo tayari</t>
+        </is>
+      </c>
+      <c r="I467" s="14" t="inlineStr"/>
+    </row>
+    <row r="468" ht="44" customHeight="1">
+      <c r="A468" s="11" t="inlineStr">
+        <is>
+          <t>setup_channels_help</t>
+        </is>
+      </c>
+      <c r="B468" s="11" t="inlineStr">
+        <is>
+          <t>Read by bank staff, not customers. Keep it short — it has to fit the same space as the English. Use the words your branch staff already use.</t>
+        </is>
+      </c>
+      <c r="C468" s="11" t="inlineStr">
+        <is>
+          <t>The website widget is already live. Telegram takes about a minute and needs nobody's approval.</t>
+        </is>
+      </c>
+      <c r="D468" s="12" t="inlineStr">
+        <is>
+          <t>የድረ-ገጽ መሣሪያው አስቀድሞ ሠርቷል። ቴሌግራም አንድ ደቂቃ ያህል ይወስዳል፣ የማንም ፈቃድ አይፈልግም።</t>
+        </is>
+      </c>
+      <c r="E468" s="13" t="inlineStr">
+        <is>
+          <t>Meeshaan marsariitii duraanuu hojjechaa jira. Telegram daqiiqaa tokko fudhata, eeyyama nama kamiyyuu hin barbaadu.</t>
+        </is>
+      </c>
+      <c r="F468" s="12" t="inlineStr">
+        <is>
+          <t>እቲ ናይ መርበብ ሓበሬታ መሳርሒ ድሮ ይሰርሕ ኣሎ። ተለግራም ሓደ ደቒቕ ይወስድ፡ ፍቓድ ናይ ዝኾነ ኣየድልዮን።</t>
+        </is>
+      </c>
+      <c r="G468" s="13" t="inlineStr">
+        <is>
+          <t>Qalabka websaydhku horeba wuu shaqeynayaa. Telegram wuxuu qaataa ilaa daqiiqad, oo ogolaansho cidna uma baahna.</t>
+        </is>
+      </c>
+      <c r="H468" s="13" t="inlineStr">
+        <is>
+          <t>Kifaa cha tovuti tayari kinafanya kazi. Telegram huchukua kama dakika moja na hakihitaji idhini ya mtu.</t>
+        </is>
+      </c>
+      <c r="I468" s="14" t="inlineStr"/>
+    </row>
+    <row r="469" ht="44" customHeight="1">
+      <c r="A469" s="11" t="inlineStr">
+        <is>
+          <t>setup_team</t>
+        </is>
+      </c>
+      <c r="B469" s="11" t="inlineStr">
+        <is>
+          <t>Read by bank staff, not customers. Keep it short — it has to fit the same space as the English. Use the words your branch staff already use.</t>
+        </is>
+      </c>
+      <c r="C469" s="11" t="inlineStr">
+        <is>
+          <t>Bring your colleagues in</t>
+        </is>
+      </c>
+      <c r="D469" s="12" t="inlineStr">
+        <is>
+          <t>ባልደረቦችዎን ያስገቡ</t>
+        </is>
+      </c>
+      <c r="E469" s="13" t="inlineStr">
+        <is>
+          <t>Hojjettoota hiriyoota kee galchi</t>
+        </is>
+      </c>
+      <c r="F469" s="12" t="inlineStr">
+        <is>
+          <t>ንመሳርሕትኻ ኣእቱ</t>
+        </is>
+      </c>
+      <c r="G469" s="13" t="inlineStr">
+        <is>
+          <t>Asxaabtaada shaqada soo gali</t>
+        </is>
+      </c>
+      <c r="H469" s="13" t="inlineStr">
+        <is>
+          <t>Waingize wenzako</t>
+        </is>
+      </c>
+      <c r="I469" s="14" t="inlineStr"/>
+    </row>
+    <row r="470" ht="44" customHeight="1">
+      <c r="A470" s="11" t="inlineStr">
+        <is>
+          <t>setup_team_help</t>
+        </is>
+      </c>
+      <c r="B470" s="11" t="inlineStr">
+        <is>
+          <t>Read by bank staff, not customers. Keep it short — it has to fit the same space as the English. Use the words your branch staff already use.</t>
+        </is>
+      </c>
+      <c r="C470" s="11" t="inlineStr">
+        <is>
+          <t>Whoever answers escalations needs their own sign-in, not a shared one.</t>
+        </is>
+      </c>
+      <c r="D470" s="12" t="inlineStr">
+        <is>
+          <t>ጥያቄዎችን የሚመልሱ ሰዎች የየራሳቸው መግቢያ ያስፈልጋቸዋል፣ የጋራ አይደለም።</t>
+        </is>
+      </c>
+      <c r="E470" s="13" t="inlineStr">
+        <is>
+          <t>Namni gaaffii deebisu seensa mataa isaa qabaachuu qaba, kan waliin qooddamu miti.</t>
+        </is>
+      </c>
+      <c r="F470" s="12" t="inlineStr">
+        <is>
+          <t>ነቲ ናብ ሰብ ዝመሓላለፍ ዝምልስ ሰብ ናይ ገዛእ ርእሱ መእተዊ የድልዮ፡ ናይ ሓባር ዘይኮነ።</t>
+        </is>
+      </c>
+      <c r="G470" s="13" t="inlineStr">
+        <is>
+          <t>Qofka ka jawaabaya kordhinta wuxuu u baahan yahay gelitaan u gaar ah, ee ma aha mid la wadaago.</t>
+        </is>
+      </c>
+      <c r="H470" s="13" t="inlineStr">
+        <is>
+          <t>Yeyote anayejibu maswali yaliyopandishwa anahitaji kuingia kwake mwenyewe, si kwa pamoja.</t>
+        </is>
+      </c>
+      <c r="I470" s="14" t="inlineStr"/>
+    </row>
+    <row r="471" ht="44" customHeight="1">
+      <c r="A471" s="11" t="inlineStr">
+        <is>
+          <t>setup_open</t>
+        </is>
+      </c>
+      <c r="B471" s="11" t="inlineStr">
+        <is>
+          <t>Read by bank staff, not customers. Keep it short — it has to fit the same space as the English. Use the words your branch staff already use.</t>
+        </is>
+      </c>
+      <c r="C471" s="11" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="D471" s="12" t="inlineStr">
+        <is>
+          <t>ክፈት</t>
+        </is>
+      </c>
+      <c r="E471" s="13" t="inlineStr">
+        <is>
+          <t>Bani</t>
+        </is>
+      </c>
+      <c r="F471" s="12" t="inlineStr">
+        <is>
+          <t>ክፈት</t>
+        </is>
+      </c>
+      <c r="G471" s="13" t="inlineStr">
+        <is>
+          <t>Fur</t>
+        </is>
+      </c>
+      <c r="H471" s="13" t="inlineStr">
+        <is>
+          <t>Fungua</t>
+        </is>
+      </c>
+      <c r="I471" s="14" t="inlineStr"/>
+    </row>
+    <row r="472" ht="44" customHeight="1">
+      <c r="A472" s="11" t="inlineStr">
+        <is>
+          <t>setup_step_done</t>
+        </is>
+      </c>
+      <c r="B472" s="11" t="inlineStr">
+        <is>
+          <t>Read by bank staff, not customers. Keep it short — it has to fit the same space as the English. Use the words your branch staff already use.</t>
+        </is>
+      </c>
+      <c r="C472" s="11" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="D472" s="12" t="inlineStr">
+        <is>
+          <t>ተጠናቋል</t>
+        </is>
+      </c>
+      <c r="E472" s="13" t="inlineStr">
+        <is>
+          <t>Xumurameera</t>
+        </is>
+      </c>
+      <c r="F472" s="12" t="inlineStr">
+        <is>
+          <t>ተዛዚሙ</t>
+        </is>
+      </c>
+      <c r="G472" s="13" t="inlineStr">
+        <is>
+          <t>Waa dhammaatay</t>
+        </is>
+      </c>
+      <c r="H472" s="13" t="inlineStr">
+        <is>
+          <t>Imekamilika</t>
+        </is>
+      </c>
+      <c r="I472" s="14" t="inlineStr"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:I459"/>
+  <autoFilter ref="A1:I472"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
fix: the admin panel is usable on a phone, and every surface has a mark (#177)
Below 980px the sidebar kept its markup and lost its column, so
twenty-one nav items stacked above the page and a phone scrolled about
450px before reaching the dashboard. It is a drawer now: off-canvas,
transform rather than left, closing on navigation, scrim, Escape and a
resize back to desktop. The desktop icon rail is neutralised inside it.

Two cascade bugs found by driving it at 390px: the base .navtoggle rule
sat after the breakpoint that turns it on, so the drawer had no opener
at all; and the scrim's media rule set position without restating
display, so it opened with nothing dimming the page.

Also serves a favicon at both paths — every surface 404'd and showed a
blank tab. It is the mark site.html already carried inline, not a new
one.

nav_menu in six languages; workbook regenerated.
</commit_message>
<xml_diff>
--- a/review/Olink_Bank_Assist_language_review.xlsx
+++ b/review/Olink_Bank_Assist_language_review.xlsx
@@ -17,7 +17,7 @@
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'1. What the assistant says'!$A$1:$I$24</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'2. What it understands'!$A$1:$E$91</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'3. Buttons customers see'!$A$1:$I$53</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'4. The staff panel'!$A$1:$I$472</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'4. The staff panel'!$A$1:$I$473</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -752,7 +752,7 @@
       </c>
       <c r="C26" s="6" t="inlineStr">
         <is>
-          <t>546 strings in 5 languages</t>
+          <t>547 strings in 5 languages</t>
         </is>
       </c>
     </row>
@@ -6345,7 +6345,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I472"/>
+  <dimension ref="A1:I473"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
@@ -26659,8 +26659,51 @@
       </c>
       <c r="I472" s="14" t="inlineStr"/>
     </row>
+    <row r="473" ht="44" customHeight="1">
+      <c r="A473" s="11" t="inlineStr">
+        <is>
+          <t>nav_menu</t>
+        </is>
+      </c>
+      <c r="B473" s="11" t="inlineStr">
+        <is>
+          <t>Read by bank staff, not customers. Keep it short — it has to fit the same space as the English. Use the words your branch staff already use.</t>
+        </is>
+      </c>
+      <c r="C473" s="11" t="inlineStr">
+        <is>
+          <t>Menu</t>
+        </is>
+      </c>
+      <c r="D473" s="12" t="inlineStr">
+        <is>
+          <t>ዝርዝር</t>
+        </is>
+      </c>
+      <c r="E473" s="13" t="inlineStr">
+        <is>
+          <t>Baafata</t>
+        </is>
+      </c>
+      <c r="F473" s="12" t="inlineStr">
+        <is>
+          <t>ዝርዝር</t>
+        </is>
+      </c>
+      <c r="G473" s="13" t="inlineStr">
+        <is>
+          <t>Liiska</t>
+        </is>
+      </c>
+      <c r="H473" s="13" t="inlineStr">
+        <is>
+          <t>Menyu</t>
+        </is>
+      </c>
+      <c r="I473" s="14" t="inlineStr"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:I472"/>
+  <autoFilter ref="A1:I473"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>